<commit_message>
Integrar mejor estructura para el proyecto y definicion de variables estacionales
Cambios traídos desde (9f96358ab9f23d81231cb1b3dc0deaaae5b6ef94)
</commit_message>
<xml_diff>
--- a/data/Data estacionaria.xlsx
+++ b/data/Data estacionaria.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Mi unidad\ANTES 2026\INVESTIGACION\INVESTIGACIÓN EXTERNA\UDEP\TESIS ECONOMETRICA\TRATADO DE DATOS\Datos procesados\contrafactual\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\econometria-udep\econometria-app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C736EEE5-2791-4CE2-AC6A-155DF85BD982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5442C062-C4A7-42CB-A234-411F122C9275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2325" yWindow="1335" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Hoja1!$A$1:$D$253</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -3957,6 +3957,7 @@
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
     <col min="10" max="10" width="18.28515625" customWidth="1"/>
     <col min="11" max="11" width="19.5703125" customWidth="1"/>
     <col min="13" max="13" width="25.5703125" customWidth="1"/>
@@ -4084,7 +4085,7 @@
         <v>423.84500000000003</v>
       </c>
       <c r="I2">
-        <v>7.3503285399143553E-2</v>
+        <v>7.3503285399143595E-2</v>
       </c>
       <c r="J2">
         <v>803.90099999999995</v>
@@ -4143,13 +4144,13 @@
         <v>429.81599999999997</v>
       </c>
       <c r="I3">
-        <v>7.6065106929476795E-2</v>
+        <v>7.4023393546291449E-2</v>
       </c>
       <c r="J3">
         <v>815.74099999999999</v>
       </c>
       <c r="K3">
-        <v>5.8606837219166381E-2</v>
+        <v>5.7207578214369927E-2</v>
       </c>
       <c r="L3">
         <v>3.5</v>
@@ -4238,13 +4239,13 @@
         <v>445.13900000000001</v>
       </c>
       <c r="I4">
-        <v>7.9009028640492071E-2</v>
+        <v>7.6362555035765653E-2</v>
       </c>
       <c r="J4">
         <v>839.89200000000005</v>
       </c>
       <c r="K4">
-        <v>6.1017368899810923E-2</v>
+        <v>5.9231655938548573E-2</v>
       </c>
       <c r="L4">
         <v>3</v>
@@ -4333,13 +4334,13 @@
         <v>456.49599999999998</v>
       </c>
       <c r="I5">
-        <v>7.8024780063790267E-2</v>
+        <v>7.3923348040563136E-2</v>
       </c>
       <c r="J5">
         <v>861.851</v>
       </c>
       <c r="K5">
-        <v>5.9614712984030878E-2</v>
+        <v>5.6902517788027761E-2</v>
       </c>
       <c r="L5">
         <v>3</v>
@@ -4428,13 +4429,13 @@
         <v>471.23599999999999</v>
       </c>
       <c r="I6">
-        <v>7.6566730894923149E-2</v>
+        <v>7.2218557598468902E-2</v>
       </c>
       <c r="J6">
         <v>892.58999999999992</v>
       </c>
       <c r="K6">
-        <v>5.8862411633560763E-2</v>
+        <v>5.584307338801648E-2</v>
       </c>
       <c r="L6">
         <v>3</v>
@@ -4523,13 +4524,13 @@
         <v>483.49799999999999</v>
       </c>
       <c r="I7">
-        <v>7.5199897414260253E-2</v>
+        <v>7.2273461171468351E-2</v>
       </c>
       <c r="J7">
         <v>920.5630000000001</v>
       </c>
       <c r="K7">
-        <v>5.7063992361196351E-2</v>
+        <v>5.5352034549793393E-2</v>
       </c>
       <c r="L7">
         <v>3</v>
@@ -4618,13 +4619,13 @@
         <v>502.80700000000002</v>
       </c>
       <c r="I8">
-        <v>7.1470763135755858E-2</v>
+        <v>6.8053104704699274E-2</v>
       </c>
       <c r="J8">
         <v>955.93200000000002</v>
       </c>
       <c r="K8">
-        <v>5.5322972763753073E-2</v>
+        <v>5.2880499407597648E-2</v>
       </c>
       <c r="L8">
         <v>3.25</v>
@@ -4713,13 +4714,13 @@
         <v>520.96699999999998</v>
       </c>
       <c r="I9">
-        <v>6.7952480675359472E-2</v>
+        <v>6.4814751285861408E-2</v>
       </c>
       <c r="J9">
         <v>1003.971</v>
       </c>
       <c r="K9">
-        <v>5.1652886388152637E-2</v>
+        <v>4.9629812054326712E-2</v>
       </c>
       <c r="L9">
         <v>3.25</v>
@@ -4808,13 +4809,13 @@
         <v>538.88900000000001</v>
       </c>
       <c r="I10">
-        <v>6.6154625535128755E-2</v>
+        <v>6.4180529390678559E-2</v>
       </c>
       <c r="J10">
         <v>1052.442</v>
       </c>
       <c r="K10">
-        <v>4.9702501420505828E-2</v>
+        <v>4.8844747113439953E-2</v>
       </c>
       <c r="L10">
         <v>3.75</v>
@@ -4903,13 +4904,13 @@
         <v>560.404</v>
       </c>
       <c r="I11">
-        <v>6.5879258534914095E-2</v>
+        <v>6.4025358702307647E-2</v>
       </c>
       <c r="J11">
         <v>1107.1030000000001</v>
       </c>
       <c r="K11">
-        <v>4.7281960215083872E-2</v>
+        <v>4.6537077827255302E-2</v>
       </c>
       <c r="L11">
         <v>4.75</v>
@@ -4998,13 +4999,13 @@
         <v>577.70699999999999</v>
       </c>
       <c r="I12">
-        <v>6.2645943358830697E-2</v>
+        <v>6.3271307814498703E-2</v>
       </c>
       <c r="J12">
         <v>1146.173</v>
       </c>
       <c r="K12">
-        <v>4.5588231444991287E-2</v>
+        <v>4.6557953971036001E-2</v>
       </c>
       <c r="L12">
         <v>4.75</v>
@@ -5093,13 +5094,13 @@
         <v>593.23599999999999</v>
       </c>
       <c r="I13">
-        <v>5.721837514918178E-2</v>
+        <v>6.3245363725760992E-2</v>
       </c>
       <c r="J13">
         <v>1184.2249999999999</v>
       </c>
       <c r="K13">
-        <v>4.1618780214908488E-2</v>
+        <v>4.6923570223188153E-2</v>
       </c>
       <c r="L13">
         <v>4.5</v>
@@ -5283,13 +5284,13 @@
         <v>604.05600000000004</v>
       </c>
       <c r="I15">
-        <v>6.2749149085515252E-2</v>
+        <v>6.0707435702329907E-2</v>
       </c>
       <c r="J15">
         <v>1230.4649999999999</v>
       </c>
       <c r="K15">
-        <v>4.6232115501050421E-2</v>
+        <v>4.4832856496253973E-2</v>
       </c>
       <c r="L15">
         <v>4.25</v>
@@ -5378,13 +5379,13 @@
         <v>626.01</v>
       </c>
       <c r="I16">
-        <v>6.5203431255091773E-2</v>
+        <v>6.2556957650365355E-2</v>
       </c>
       <c r="J16">
         <v>1272.1199999999999</v>
       </c>
       <c r="K16">
-        <v>4.7859478665534708E-2</v>
+        <v>4.6073765704272358E-2</v>
       </c>
       <c r="L16">
         <v>4.25</v>
@@ -5473,13 +5474,13 @@
         <v>638.35299999999995</v>
       </c>
       <c r="I17">
-        <v>6.6718571072745023E-2</v>
+        <v>6.2617139049517892E-2</v>
       </c>
       <c r="J17">
         <v>1296.5440000000001</v>
       </c>
       <c r="K17">
-        <v>4.8955531011674117E-2</v>
+        <v>4.6243335815670999E-2</v>
       </c>
       <c r="L17">
         <v>4.25</v>
@@ -5568,13 +5569,13 @@
         <v>655.45899999999995</v>
       </c>
       <c r="I18">
-        <v>6.7432135343324304E-2</v>
+        <v>6.3083962046870057E-2</v>
       </c>
       <c r="J18">
         <v>1326.8409999999999</v>
       </c>
       <c r="K18">
-        <v>4.9776122383917903E-2</v>
+        <v>4.6756784138373621E-2</v>
       </c>
       <c r="L18">
         <v>4.25</v>
@@ -5663,13 +5664,13 @@
         <v>667.43100000000004</v>
       </c>
       <c r="I19">
-        <v>6.7238411161603215E-2</v>
+        <v>6.4311974918811313E-2</v>
       </c>
       <c r="J19">
         <v>1349.962</v>
       </c>
       <c r="K19">
-        <v>5.0239191917994717E-2</v>
+        <v>4.8527234106591759E-2</v>
       </c>
       <c r="L19">
         <v>4.25</v>
@@ -5758,13 +5759,13 @@
         <v>683.72900000000004</v>
       </c>
       <c r="I20">
-        <v>6.6233844110751477E-2</v>
+        <v>6.2816185679694894E-2</v>
       </c>
       <c r="J20">
         <v>1378.318</v>
       </c>
       <c r="K20">
-        <v>4.9513247305774201E-2</v>
+        <v>4.7070773949618783E-2</v>
       </c>
       <c r="L20">
         <v>4</v>
@@ -5853,13 +5854,13 @@
         <v>702.43100000000004</v>
       </c>
       <c r="I21">
-        <v>6.7380283615045458E-2</v>
+        <v>6.4242554225547394E-2</v>
       </c>
       <c r="J21">
         <v>1419.5039999999999</v>
       </c>
       <c r="K21">
-        <v>5.003156031966096E-2</v>
+        <v>4.8008485985835028E-2</v>
       </c>
       <c r="L21">
         <v>3.5</v>
@@ -5948,13 +5949,13 @@
         <v>722.02599999999995</v>
       </c>
       <c r="I22">
-        <v>6.8606947672244498E-2</v>
+        <v>6.6632851527794301E-2</v>
       </c>
       <c r="J22">
         <v>1464.114</v>
       </c>
       <c r="K22">
-        <v>5.0136806286942143E-2</v>
+        <v>4.9279051979876261E-2</v>
       </c>
       <c r="L22">
         <v>2.75</v>
@@ -6043,13 +6044,13 @@
         <v>756.31000000000006</v>
       </c>
       <c r="I23">
-        <v>6.5988814110616009E-2</v>
+        <v>6.4134914278009561E-2</v>
       </c>
       <c r="J23">
         <v>1515.5429999999999</v>
       </c>
       <c r="K23">
-        <v>4.8925038748488157E-2</v>
+        <v>4.818015636065958E-2</v>
       </c>
       <c r="L23">
         <v>2.75</v>
@@ -6138,13 +6139,13 @@
         <v>805.49299999999994</v>
       </c>
       <c r="I24">
-        <v>6.1624371658102563E-2</v>
+        <v>6.2249736113770583E-2</v>
       </c>
       <c r="J24">
         <v>1580.4380000000001</v>
       </c>
       <c r="K24">
-        <v>4.7088212255083722E-2</v>
+        <v>4.8057934781128443E-2</v>
       </c>
       <c r="L24">
         <v>2.5</v>
@@ -6233,13 +6234,13 @@
         <v>830.68899999999996</v>
       </c>
       <c r="I25">
-        <v>5.8020510684504083E-2</v>
+        <v>6.4047499261083302E-2</v>
       </c>
       <c r="J25">
         <v>1623.732</v>
       </c>
       <c r="K25">
-        <v>4.35441316670485E-2</v>
+        <v>4.8848921675328158E-2</v>
       </c>
       <c r="L25">
         <v>2.5</v>
@@ -6423,13 +6424,13 @@
         <v>854.36400000000003</v>
       </c>
       <c r="I27">
-        <v>6.6966772944552902E-2</v>
+        <v>6.4925059561367557E-2</v>
       </c>
       <c r="J27">
         <v>1672.02</v>
       </c>
       <c r="K27">
-        <v>5.0061004054975419E-2</v>
+        <v>4.8661745050178958E-2</v>
       </c>
       <c r="L27">
         <v>2.5</v>
@@ -6518,13 +6519,13 @@
         <v>891.87099999999998</v>
       </c>
       <c r="I28">
-        <v>6.8156717731600203E-2</v>
+        <v>6.5510244126873785E-2</v>
       </c>
       <c r="J28">
         <v>1725.3879999999999</v>
       </c>
       <c r="K28">
-        <v>5.0915504222818292E-2</v>
+        <v>4.9129791261555943E-2</v>
       </c>
       <c r="L28">
         <v>2.5</v>
@@ -6613,13 +6614,13 @@
         <v>913.06500000000005</v>
       </c>
       <c r="I29">
-        <v>7.1071610454896419E-2</v>
+        <v>6.6970178431669289E-2</v>
       </c>
       <c r="J29">
         <v>1756.796</v>
       </c>
       <c r="K29">
-        <v>5.2440920858198667E-2</v>
+        <v>4.972872566219555E-2</v>
       </c>
       <c r="L29">
         <v>2.5</v>
@@ -6708,13 +6709,13 @@
         <v>932.97</v>
       </c>
       <c r="I30">
-        <v>7.0522096101696727E-2</v>
+        <v>6.617392280524248E-2</v>
       </c>
       <c r="J30">
         <v>1775.136</v>
       </c>
       <c r="K30">
-        <v>5.310691687848143E-2</v>
+        <v>5.0087578632937148E-2</v>
       </c>
       <c r="L30">
         <v>2.5</v>
@@ -6803,13 +6804,13 @@
         <v>949.41100000000006</v>
       </c>
       <c r="I31">
-        <v>7.5842812017134831E-2</v>
+        <v>7.2916375774342929E-2</v>
       </c>
       <c r="J31">
         <v>1798.509</v>
       </c>
       <c r="K31">
-        <v>5.6031412686842273E-2</v>
+        <v>5.4319454875439308E-2</v>
       </c>
       <c r="L31">
         <v>2.5</v>
@@ -6898,13 +6899,13 @@
         <v>961.62199999999996</v>
       </c>
       <c r="I32">
-        <v>7.8350952869214716E-2</v>
+        <v>7.4933294438158132E-2</v>
       </c>
       <c r="J32">
         <v>1806.241</v>
       </c>
       <c r="K32">
-        <v>5.8428526425875621E-2</v>
+        <v>5.5986053069720203E-2</v>
       </c>
       <c r="L32">
         <v>2.5</v>
@@ -6993,13 +6994,13 @@
         <v>980.64400000000001</v>
       </c>
       <c r="I33">
-        <v>7.7140124244883979E-2</v>
+        <v>7.4002394855385914E-2</v>
       </c>
       <c r="J33">
         <v>1832.4179999999999</v>
       </c>
       <c r="K33">
-        <v>5.7651147281897457E-2</v>
+        <v>5.5628072948071518E-2</v>
       </c>
       <c r="L33">
         <v>2.75</v>
@@ -7088,13 +7089,13 @@
         <v>1007.597</v>
       </c>
       <c r="I34">
-        <v>7.4039521753240634E-2</v>
+        <v>7.2065425608790437E-2</v>
       </c>
       <c r="J34">
         <v>1878.732</v>
       </c>
       <c r="K34">
-        <v>5.5087154527628211E-2</v>
+        <v>5.4229400220562329E-2</v>
       </c>
       <c r="L34">
         <v>2.75</v>
@@ -7183,13 +7184,13 @@
         <v>1024.7460000000001</v>
       </c>
       <c r="I35">
-        <v>7.1483079709508485E-2</v>
+        <v>6.9629179876902036E-2</v>
       </c>
       <c r="J35">
         <v>1915.915</v>
       </c>
       <c r="K35">
-        <v>5.4248753206692368E-2</v>
+        <v>5.3503870818863791E-2</v>
       </c>
       <c r="L35">
         <v>3</v>
@@ -7278,13 +7279,13 @@
         <v>1069.412</v>
       </c>
       <c r="I36">
-        <v>6.8590028913084938E-2</v>
+        <v>6.9215393368752945E-2</v>
       </c>
       <c r="J36">
         <v>1992.28</v>
       </c>
       <c r="K36">
-        <v>5.1585620495111117E-2</v>
+        <v>5.2555343021155831E-2</v>
       </c>
       <c r="L36">
         <v>3</v>
@@ -7373,13 +7374,13 @@
         <v>1111.04079688</v>
       </c>
       <c r="I37">
-        <v>6.8279505849859035E-2</v>
+        <v>7.4306494426438247E-2</v>
       </c>
       <c r="J37">
         <v>2066.3907967099999</v>
       </c>
       <c r="K37">
-        <v>5.0199225318441933E-2</v>
+        <v>5.5504015326721598E-2</v>
       </c>
       <c r="L37">
         <v>3</v>
@@ -7563,13 +7564,13 @@
         <v>1118.2339999999999</v>
       </c>
       <c r="I39">
-        <v>7.9680102733417163E-2</v>
+        <v>7.7638389350231818E-2</v>
       </c>
       <c r="J39">
         <v>2100.4059999999999</v>
       </c>
       <c r="K39">
-        <v>5.8464411166222148E-2</v>
+        <v>5.7065152161425693E-2</v>
       </c>
       <c r="L39">
         <v>3</v>
@@ -7658,13 +7659,13 @@
         <v>1141.2049999999999</v>
       </c>
       <c r="I40">
-        <v>7.9558011049723765E-2</v>
+        <v>7.6911537444997347E-2</v>
       </c>
       <c r="J40">
         <v>2149.7139999999999</v>
       </c>
       <c r="K40">
-        <v>5.7869558462195443E-2</v>
+        <v>5.6083845500933087E-2</v>
       </c>
       <c r="L40">
         <v>3</v>
@@ -7753,13 +7754,13 @@
         <v>1168.1579999999999</v>
       </c>
       <c r="I41">
-        <v>8.0398370768337862E-2</v>
+        <v>7.6296938745110732E-2</v>
       </c>
       <c r="J41">
         <v>2191.56</v>
       </c>
       <c r="K41">
-        <v>5.8077351293142787E-2</v>
+        <v>5.536515609713967E-2</v>
       </c>
       <c r="L41">
         <v>3</v>
@@ -7848,13 +7849,13 @@
         <v>1182.146</v>
       </c>
       <c r="I42">
-        <v>8.0909633835414579E-2</v>
+        <v>7.6561460538960333E-2</v>
       </c>
       <c r="J42">
         <v>2218.1990000000001</v>
       </c>
       <c r="K42">
-        <v>5.8635857287826748E-2</v>
+        <v>5.5616519042282472E-2</v>
       </c>
       <c r="L42">
         <v>3</v>
@@ -7943,13 +7944,13 @@
         <v>1191.4269999999999</v>
       </c>
       <c r="I43">
-        <v>7.7644706725632354E-2</v>
+        <v>7.4718270482840451E-2</v>
       </c>
       <c r="J43">
         <v>2253.0819999999999</v>
       </c>
       <c r="K43">
-        <v>5.602547976505072E-2</v>
+        <v>5.4313521953647761E-2</v>
       </c>
       <c r="L43">
         <v>3</v>
@@ -8038,13 +8039,13 @@
         <v>1208.9159999999999</v>
       </c>
       <c r="I44">
-        <v>7.9357043831002325E-2</v>
+        <v>7.5939385399945741E-2</v>
       </c>
       <c r="J44">
         <v>2299.2640000000001</v>
       </c>
       <c r="K44">
-        <v>5.674859433279518E-2</v>
+        <v>5.4306120976639748E-2</v>
       </c>
       <c r="L44">
         <v>3</v>
@@ -8133,13 +8134,13 @@
         <v>1234.9349999999999</v>
       </c>
       <c r="I45">
-        <v>7.6269601234073059E-2</v>
+        <v>7.3131871844574994E-2</v>
       </c>
       <c r="J45">
         <v>2361.2910000000002</v>
       </c>
       <c r="K45">
-        <v>5.5082156328889582E-2</v>
+        <v>5.3059081995063651E-2</v>
       </c>
       <c r="L45">
         <v>3</v>
@@ -8228,13 +8229,13 @@
         <v>1272.1969999999999</v>
       </c>
       <c r="I46">
-        <v>7.5041837073975187E-2</v>
+        <v>7.3067740929524991E-2</v>
       </c>
       <c r="J46">
         <v>2441.98</v>
       </c>
       <c r="K46">
-        <v>5.4289142417218807E-2</v>
+        <v>5.3431388110152918E-2</v>
       </c>
       <c r="L46">
         <v>3</v>
@@ -8323,13 +8324,13 @@
         <v>1311.17</v>
       </c>
       <c r="I47">
-        <v>7.4235225028028387E-2</v>
+        <v>7.2381325195421939E-2</v>
       </c>
       <c r="J47">
         <v>2514.0650000000001</v>
       </c>
       <c r="K47">
-        <v>5.4030027067717028E-2</v>
+        <v>5.3285144679888451E-2</v>
       </c>
       <c r="L47">
         <v>3</v>
@@ -8418,13 +8419,13 @@
         <v>1365.585</v>
       </c>
       <c r="I48">
-        <v>6.9029756477992948E-2</v>
+        <v>6.9655120933660955E-2</v>
       </c>
       <c r="J48">
         <v>2607.4549999999999</v>
       </c>
       <c r="K48">
-        <v>5.0183799912174899E-2</v>
+        <v>5.1153522438219613E-2</v>
       </c>
       <c r="L48">
         <v>3</v>
@@ -8513,13 +8514,13 @@
         <v>1408.7850000000001</v>
       </c>
       <c r="I49">
-        <v>6.2186919934553532E-2</v>
+        <v>6.8213908511132737E-2</v>
       </c>
       <c r="J49">
         <v>2681.643</v>
       </c>
       <c r="K49">
-        <v>4.6471510189835107E-2</v>
+        <v>5.1776300198114772E-2</v>
       </c>
       <c r="L49">
         <v>3.25</v>
@@ -8703,13 +8704,13 @@
         <v>1424.1969999999999</v>
       </c>
       <c r="I51">
-        <v>7.0021211953121651E-2</v>
+        <v>6.7979498569936306E-2</v>
       </c>
       <c r="J51">
         <v>2708.942</v>
       </c>
       <c r="K51">
-        <v>5.2947977476077372E-2</v>
+        <v>5.1548718471280917E-2</v>
       </c>
       <c r="L51">
         <v>3.75</v>
@@ -8798,13 +8799,13 @@
         <v>1472.2570000000001</v>
       </c>
       <c r="I52">
-        <v>6.8541022389433368E-2</v>
+        <v>6.5894548784706949E-2</v>
       </c>
       <c r="J52">
         <v>2783.2559999999999</v>
       </c>
       <c r="K52">
-        <v>5.2161569040002083E-2</v>
+        <v>5.0375856078739727E-2</v>
       </c>
       <c r="L52">
         <v>4</v>
@@ -8893,13 +8894,13 @@
         <v>1478.075</v>
       </c>
       <c r="I53">
-        <v>6.8999205047105189E-2</v>
+        <v>6.4897773023878058E-2</v>
       </c>
       <c r="J53">
         <v>2798.692</v>
       </c>
       <c r="K53">
-        <v>5.3649347623818552E-2</v>
+        <v>5.0937152427815442E-2</v>
       </c>
       <c r="L53">
         <v>4.25</v>
@@ -8988,13 +8989,13 @@
         <v>1498.213</v>
       </c>
       <c r="I54">
-        <v>6.9127687451650738E-2</v>
+        <v>6.4779514155196491E-2</v>
       </c>
       <c r="J54">
         <v>2842.3690000000001</v>
       </c>
       <c r="K54">
-        <v>5.3169029073987233E-2</v>
+        <v>5.014969082844295E-2</v>
       </c>
       <c r="L54">
         <v>4.5</v>
@@ -9083,13 +9084,13 @@
         <v>1514.933</v>
       </c>
       <c r="I55">
-        <v>6.8843968677162623E-2</v>
+        <v>6.5917532434370721E-2</v>
       </c>
       <c r="J55">
         <v>2867.7020000000002</v>
       </c>
       <c r="K55">
-        <v>5.2633781334322748E-2</v>
+        <v>5.0921823522919789E-2</v>
       </c>
       <c r="L55">
         <v>4.5</v>
@@ -9178,13 +9179,13 @@
         <v>1526.9110000000001</v>
       </c>
       <c r="I56">
-        <v>6.9224728880727171E-2</v>
+        <v>6.5807070449670588E-2</v>
       </c>
       <c r="J56">
         <v>2902.9949999999999</v>
       </c>
       <c r="K56">
-        <v>5.3122723256498902E-2</v>
+        <v>5.0680249900343477E-2</v>
       </c>
       <c r="L56">
         <v>4.5</v>
@@ -9273,13 +9274,13 @@
         <v>1559.5129999999999</v>
       </c>
       <c r="I57">
-        <v>6.882404955906106E-2</v>
+        <v>6.5686320169562995E-2</v>
       </c>
       <c r="J57">
         <v>2978.0120000000002</v>
       </c>
       <c r="K57">
-        <v>5.2362112711433012E-2</v>
+        <v>5.033903837760708E-2</v>
       </c>
       <c r="L57">
         <v>4.5</v>
@@ -9368,13 +9369,13 @@
         <v>1592.5260000000001</v>
       </c>
       <c r="I58">
-        <v>6.8556494525050138E-2</v>
+        <v>6.6582398380599941E-2</v>
       </c>
       <c r="J58">
         <v>3073.47</v>
       </c>
       <c r="K58">
-        <v>5.1024412146531438E-2</v>
+        <v>5.0166657839465563E-2</v>
       </c>
       <c r="L58">
         <v>4.5</v>
@@ -9463,13 +9464,13 @@
         <v>1639.186864</v>
       </c>
       <c r="I59">
-        <v>6.8635800146334011E-2</v>
+        <v>6.6781900313727563E-2</v>
       </c>
       <c r="J59">
         <v>3154.2887730000002</v>
       </c>
       <c r="K59">
-        <v>5.1437089523572288E-2</v>
+        <v>5.0692207135743711E-2</v>
       </c>
       <c r="L59">
         <v>4.5</v>
@@ -9558,13 +9559,13 @@
         <v>1697.2960840000001</v>
       </c>
       <c r="I60">
-        <v>6.4058838068938834E-2</v>
+        <v>6.468420252460684E-2</v>
       </c>
       <c r="J60">
         <v>3250.7574420000001</v>
       </c>
       <c r="K60">
-        <v>4.9014513030529568E-2</v>
+        <v>4.9984235556574282E-2</v>
       </c>
       <c r="L60">
         <v>4.5</v>
@@ -9653,13 +9654,13 @@
         <v>1715.617872</v>
       </c>
       <c r="I61">
-        <v>5.7957466299931391E-2</v>
+        <v>6.398445487651061E-2</v>
       </c>
       <c r="J61">
         <v>3295.320012000001</v>
       </c>
       <c r="K61">
-        <v>4.3334175278877278E-2</v>
+        <v>4.8638965287156943E-2</v>
       </c>
       <c r="L61">
         <v>4.5</v>
@@ -9843,13 +9844,13 @@
         <v>1719.67299</v>
       </c>
       <c r="I63">
-        <v>6.7261969381748568E-2</v>
+        <v>6.5220255998563223E-2</v>
       </c>
       <c r="J63">
         <v>3346.8457210000001</v>
       </c>
       <c r="K63">
-        <v>4.934749067269599E-2</v>
+        <v>4.7948231667899542E-2</v>
       </c>
       <c r="L63">
         <v>4.5</v>
@@ -9938,13 +9939,13 @@
         <v>1745.3272649999999</v>
       </c>
       <c r="I64">
-        <v>6.6438672749434199E-2</v>
+        <v>6.3792199144707781E-2</v>
       </c>
       <c r="J64">
         <v>3399.4933139999998</v>
       </c>
       <c r="K64">
-        <v>4.8863007706447872E-2</v>
+        <v>4.7077294745185523E-2</v>
       </c>
       <c r="L64">
         <v>4.5</v>
@@ -10033,13 +10034,13 @@
         <v>1760.0811670000001</v>
       </c>
       <c r="I65">
-        <v>6.753625300281392E-2</v>
+        <v>6.343482097958679E-2</v>
       </c>
       <c r="J65">
         <v>3440.4792269999998</v>
       </c>
       <c r="K65">
-        <v>4.9343143439941492E-2</v>
+        <v>4.6630948243938368E-2</v>
       </c>
       <c r="L65">
         <v>4.5</v>
@@ -10128,13 +10129,13 @@
         <v>1785.299947</v>
       </c>
       <c r="I66">
-        <v>6.6856970001355182E-2</v>
+        <v>6.2508796704900935E-2</v>
       </c>
       <c r="J66">
         <v>3508.5701749999998</v>
       </c>
       <c r="K66">
-        <v>4.8499526163816857E-2</v>
+        <v>4.5480187918272567E-2</v>
       </c>
       <c r="L66">
         <v>4.5</v>
@@ -10223,13 +10224,13 @@
         <v>1802.411325</v>
       </c>
       <c r="I67">
-        <v>6.4247403682952328E-2</v>
+        <v>6.1320967440160433E-2</v>
       </c>
       <c r="J67">
         <v>3545.9625860000001</v>
       </c>
       <c r="K67">
-        <v>4.6255975640460398E-2</v>
+        <v>4.4544017829057439E-2</v>
       </c>
       <c r="L67">
         <v>4.5</v>
@@ -10318,13 +10319,13 @@
         <v>1846.8436380000001</v>
       </c>
       <c r="I68">
-        <v>6.3304075447669278E-2</v>
+        <v>5.9886417016612688E-2</v>
       </c>
       <c r="J68">
         <v>3621.2695960000001</v>
       </c>
       <c r="K68">
-        <v>4.5395481513329443E-2</v>
+        <v>4.2953008157174018E-2</v>
       </c>
       <c r="L68">
         <v>4.75</v>
@@ -10413,13 +10414,13 @@
         <v>1886.026574</v>
       </c>
       <c r="I69">
-        <v>6.3124299859414396E-2</v>
+        <v>5.9986570469916331E-2</v>
       </c>
       <c r="J69">
         <v>3698.937778</v>
       </c>
       <c r="K69">
-        <v>4.5661611018318678E-2</v>
+        <v>4.3638536684492753E-2</v>
       </c>
       <c r="L69">
         <v>4.75</v>
@@ -10508,13 +10509,13 @@
         <v>1924.0648189999999</v>
       </c>
       <c r="I70">
-        <v>6.1840581369727747E-2</v>
+        <v>5.9866485225277537E-2</v>
       </c>
       <c r="J70">
         <v>3766.832343</v>
       </c>
       <c r="K70">
-        <v>4.4638802497401188E-2</v>
+        <v>4.3781048190335313E-2</v>
       </c>
       <c r="L70">
         <v>5</v>
@@ -10603,13 +10604,13 @@
         <v>1976.5700529999999</v>
       </c>
       <c r="I71">
-        <v>6.0917456387264209E-2</v>
+        <v>5.906355655465776E-2</v>
       </c>
       <c r="J71">
         <v>3852.2062299999998</v>
       </c>
       <c r="K71">
-        <v>4.3792806752197183E-2</v>
+        <v>4.3047924364368613E-2</v>
       </c>
       <c r="L71">
         <v>5</v>
@@ -10698,13 +10699,13 @@
         <v>2055.8010490000001</v>
       </c>
       <c r="I72">
-        <v>5.5743802667939962E-2</v>
+        <v>5.6369167123607983E-2</v>
       </c>
       <c r="J72">
         <v>3984.5956160000001</v>
       </c>
       <c r="K72">
-        <v>4.0813032907779011E-2</v>
+        <v>4.1782755433823718E-2</v>
       </c>
       <c r="L72">
         <v>5</v>
@@ -10793,13 +10794,13 @@
         <v>2093.5825920000002</v>
       </c>
       <c r="I73">
-        <v>5.1939960914615779E-2</v>
+        <v>5.7966949491194991E-2</v>
       </c>
       <c r="J73">
         <v>4062.9678629999999</v>
       </c>
       <c r="K73">
-        <v>3.780482055956641E-2</v>
+        <v>4.3109610567846082E-2</v>
       </c>
       <c r="L73">
         <v>5</v>
@@ -10983,13 +10984,13 @@
         <v>2122.0239470000001</v>
       </c>
       <c r="I75">
-        <v>5.7036064164642533E-2</v>
+        <v>5.4994350781457188E-2</v>
       </c>
       <c r="J75">
         <v>4146.5667830000002</v>
       </c>
       <c r="K75">
-        <v>4.1862801947786688E-2</v>
+        <v>4.0463542942990233E-2</v>
       </c>
       <c r="L75">
         <v>5.25</v>
@@ -11078,13 +11079,13 @@
         <v>2167.6918799999999</v>
       </c>
       <c r="I76">
-        <v>6.0179218828830983E-2</v>
+        <v>5.7532745224104558E-2</v>
       </c>
       <c r="J76">
         <v>4245.6531349999996</v>
       </c>
       <c r="K76">
-        <v>4.5388602618381353E-2</v>
+        <v>4.3602889657118997E-2</v>
       </c>
       <c r="L76">
         <v>5.25</v>
@@ -11173,13 +11174,13 @@
         <v>2269.7607360000002</v>
       </c>
       <c r="I77">
-        <v>5.7888840843883557E-2</v>
+        <v>5.3787408820656427E-2</v>
       </c>
       <c r="J77">
         <v>4399.9824550000003</v>
       </c>
       <c r="K77">
-        <v>4.3868692880958307E-2</v>
+        <v>4.115649768495519E-2</v>
       </c>
       <c r="L77">
         <v>5.5</v>
@@ -11268,13 +11269,13 @@
         <v>2330.57141</v>
       </c>
       <c r="I78">
-        <v>5.7605815648446489E-2</v>
+        <v>5.3257642351992242E-2</v>
       </c>
       <c r="J78">
         <v>4526.5504179999998</v>
       </c>
       <c r="K78">
-        <v>4.4176606805222167E-2</v>
+        <v>4.1157268559677877E-2</v>
       </c>
       <c r="L78">
         <v>5.5</v>
@@ -11363,13 +11364,13 @@
         <v>2394.7625899999998</v>
       </c>
       <c r="I79">
-        <v>5.5435742379790563E-2</v>
+        <v>5.2509306136998661E-2</v>
       </c>
       <c r="J79">
         <v>4676.6022149999999</v>
       </c>
       <c r="K79">
-        <v>4.2804988065464539E-2</v>
+        <v>4.109303025406158E-2</v>
       </c>
       <c r="L79">
         <v>5.75</v>
@@ -11458,13 +11459,13 @@
         <v>2440.077123</v>
       </c>
       <c r="I80">
-        <v>5.6105219261137262E-2</v>
+        <v>5.2687560830080679E-2</v>
       </c>
       <c r="J80">
         <v>4766.5243909999999</v>
       </c>
       <c r="K80">
-        <v>4.3185111438570643E-2</v>
+        <v>4.0742638082415218E-2</v>
       </c>
       <c r="L80">
         <v>6</v>
@@ -11553,13 +11554,13 @@
         <v>2529.017875</v>
       </c>
       <c r="I81">
-        <v>5.4039079498400137E-2</v>
+        <v>5.0901350108902073E-2</v>
       </c>
       <c r="J81">
         <v>4969.8603109999985</v>
       </c>
       <c r="K81">
-        <v>4.1352618411652581E-2</v>
+        <v>3.9329544077826649E-2</v>
       </c>
       <c r="L81">
         <v>6.25</v>
@@ -11648,13 +11649,13 @@
         <v>2601.3375289999999</v>
       </c>
       <c r="I82">
-        <v>5.2636485451634747E-2</v>
+        <v>5.0662389307184537E-2</v>
       </c>
       <c r="J82">
         <v>5125.7189829999998</v>
       </c>
       <c r="K82">
-        <v>4.0623432476614187E-2</v>
+        <v>3.9765678169548298E-2</v>
       </c>
       <c r="L82">
         <v>6.5</v>
@@ -11743,13 +11744,13 @@
         <v>2711.0647589999999</v>
       </c>
       <c r="I83">
-        <v>5.2648244762935233E-2</v>
+        <v>5.0794344930328778E-2</v>
       </c>
       <c r="J83">
         <v>5326.0372900000002</v>
       </c>
       <c r="K83">
-        <v>4.08026677560119E-2</v>
+        <v>4.0057785368183323E-2</v>
       </c>
       <c r="L83">
         <v>6.5</v>
@@ -11838,13 +11839,13 @@
         <v>2832.3490539999998</v>
       </c>
       <c r="I84">
-        <v>5.2206135677795591E-2</v>
+        <v>5.2831500133463598E-2</v>
       </c>
       <c r="J84">
         <v>5520.0780080000004</v>
       </c>
       <c r="K84">
-        <v>4.0677247617620982E-2</v>
+        <v>4.1646970143665703E-2</v>
       </c>
       <c r="L84">
         <v>6.5</v>
@@ -11933,13 +11934,13 @@
         <v>2896.6231290000001</v>
       </c>
       <c r="I85">
-        <v>4.7834649462263547E-2</v>
+        <v>5.3861638038842759E-2</v>
       </c>
       <c r="J85">
         <v>5637.2790850000001</v>
       </c>
       <c r="K85">
-        <v>3.8491848235326448E-2</v>
+        <v>4.3796638243606113E-2</v>
       </c>
       <c r="L85">
         <v>6.5</v>
@@ -12123,13 +12124,13 @@
         <v>2999.1562669999998</v>
       </c>
       <c r="I87">
-        <v>5.4184233675343862E-2</v>
+        <v>5.2142520292158517E-2</v>
       </c>
       <c r="J87">
         <v>5782.4016420000007</v>
       </c>
       <c r="K87">
-        <v>4.506345669718527E-2</v>
+        <v>4.3664197692388808E-2</v>
       </c>
       <c r="L87">
         <v>6.25</v>
@@ -12218,13 +12219,13 @@
         <v>3046.1982990000001</v>
       </c>
       <c r="I88">
-        <v>5.4601890512052963E-2</v>
+        <v>5.1955416907326538E-2</v>
       </c>
       <c r="J88">
         <v>5833.4495999999999</v>
       </c>
       <c r="K88">
-        <v>4.4541814503720058E-2</v>
+        <v>4.2756101542457708E-2</v>
       </c>
       <c r="L88">
         <v>6</v>
@@ -12313,13 +12314,13 @@
         <v>3096.3306299999999</v>
       </c>
       <c r="I89">
-        <v>5.7011844371413267E-2</v>
+        <v>5.2910412348186137E-2</v>
       </c>
       <c r="J89">
         <v>5899.6513850000001</v>
       </c>
       <c r="K89">
-        <v>4.6567108981813168E-2</v>
+        <v>4.3854913785810051E-2</v>
       </c>
       <c r="L89">
         <v>5</v>
@@ -12408,13 +12409,13 @@
         <v>3145.531309</v>
       </c>
       <c r="I90">
-        <v>5.8097223027831567E-2</v>
+        <v>5.374904973137732E-2</v>
       </c>
       <c r="J90">
         <v>5980.9730159999999</v>
       </c>
       <c r="K90">
-        <v>4.7344681415964443E-2</v>
+        <v>4.432534317042016E-2</v>
       </c>
       <c r="L90">
         <v>4</v>
@@ -12503,13 +12504,13 @@
         <v>3179.6023049999999</v>
       </c>
       <c r="I91">
-        <v>5.9671647206206192E-2</v>
+        <v>5.674521096341429E-2</v>
       </c>
       <c r="J91">
         <v>6046.0968300000004</v>
       </c>
       <c r="K91">
-        <v>4.9060861798999669E-2</v>
+        <v>4.734890398759671E-2</v>
       </c>
       <c r="L91">
         <v>3</v>
@@ -12598,13 +12599,13 @@
         <v>3225.8115579999999</v>
       </c>
       <c r="I92">
-        <v>6.157050572512085E-2</v>
+        <v>5.8152847294064267E-2</v>
       </c>
       <c r="J92">
         <v>6136.1400439999998</v>
       </c>
       <c r="K92">
-        <v>5.0936687845907318E-2</v>
+        <v>4.8494214489751893E-2</v>
       </c>
       <c r="L92">
         <v>2</v>
@@ -12693,13 +12694,13 @@
         <v>3268.6422729999999</v>
       </c>
       <c r="I93">
-        <v>6.2237762963668307E-2</v>
+        <v>5.9100033574170242E-2</v>
       </c>
       <c r="J93">
         <v>6220.39282</v>
       </c>
       <c r="K93">
-        <v>5.0785323715295531E-2</v>
+        <v>4.87622493814696E-2</v>
       </c>
       <c r="L93">
         <v>1.25</v>
@@ -12788,13 +12789,13 @@
         <v>3304.2603730000001</v>
       </c>
       <c r="I94">
-        <v>6.2600244124284693E-2</v>
+        <v>6.062614797983449E-2</v>
       </c>
       <c r="J94">
         <v>6289.6108960000001</v>
       </c>
       <c r="K94">
-        <v>5.0818878669151933E-2</v>
+        <v>4.9961124362086051E-2</v>
       </c>
       <c r="L94">
         <v>1.25</v>
@@ -12883,13 +12884,13 @@
         <v>3362.6850679999998</v>
       </c>
       <c r="I95">
-        <v>6.5024122264904297E-2</v>
+        <v>6.3170222432297848E-2</v>
       </c>
       <c r="J95">
         <v>6416.8525099999997</v>
       </c>
       <c r="K95">
-        <v>5.2309331011879533E-2</v>
+        <v>5.1564448624050963E-2</v>
       </c>
       <c r="L95">
         <v>1.25</v>
@@ -12978,13 +12979,13 @@
         <v>3429.6953109999999</v>
       </c>
       <c r="I96">
-        <v>6.6017739031745723E-2</v>
+        <v>6.664310348741373E-2</v>
       </c>
       <c r="J96">
         <v>6535.4703410000002</v>
       </c>
       <c r="K96">
-        <v>5.4341974252714302E-2</v>
+        <v>5.5311696778759023E-2</v>
       </c>
       <c r="L96">
         <v>1.25</v>
@@ -13073,13 +13074,13 @@
         <v>3456.9778649999998</v>
       </c>
       <c r="I97">
-        <v>6.1827589110120033E-2</v>
+        <v>6.7854577686699252E-2</v>
       </c>
       <c r="J97">
         <v>6610.5684780000001</v>
       </c>
       <c r="K97">
-        <v>5.0706515198434637E-2</v>
+        <v>5.6011305206714303E-2</v>
       </c>
       <c r="L97">
         <v>1.25</v>
@@ -13263,13 +13264,13 @@
         <v>3472.6644339999998</v>
       </c>
       <c r="I99">
-        <v>7.2841150018239861E-2</v>
+        <v>7.0799436635054516E-2</v>
       </c>
       <c r="J99">
         <v>6649.1859160000004</v>
       </c>
       <c r="K99">
-        <v>6.1329519606111133E-2</v>
+        <v>5.9930260601314678E-2</v>
       </c>
       <c r="L99">
         <v>1.25</v>
@@ -13358,13 +13359,13 @@
         <v>3495.8816959999999</v>
       </c>
       <c r="I100">
-        <v>7.239591868614538E-2</v>
+        <v>6.9749445081418962E-2</v>
       </c>
       <c r="J100">
         <v>6725.9597240000003</v>
       </c>
       <c r="K100">
-        <v>6.0553487340507889E-2</v>
+        <v>5.876777437924554E-2</v>
       </c>
       <c r="L100">
         <v>1.25</v>
@@ -13453,13 +13454,13 @@
         <v>3535.6035999999999</v>
       </c>
       <c r="I101">
-        <v>7.557291377347844E-2</v>
+        <v>7.1471481750251309E-2</v>
       </c>
       <c r="J101">
         <v>6819.8114840000007</v>
       </c>
       <c r="K101">
-        <v>6.2304276884613069E-2</v>
+        <v>5.9592081688609952E-2</v>
       </c>
       <c r="L101">
         <v>1.25</v>
@@ -13548,13 +13549,13 @@
         <v>3575.9268630000001</v>
       </c>
       <c r="I102">
-        <v>7.6694425111904205E-2</v>
+        <v>7.2346251815449958E-2</v>
       </c>
       <c r="J102">
         <v>6912.3054920000004</v>
       </c>
       <c r="K102">
-        <v>6.3043704955510094E-2</v>
+        <v>6.0024366709965811E-2</v>
       </c>
       <c r="L102">
         <v>1.5</v>
@@ -13643,13 +13644,13 @@
         <v>3584.3366620000002</v>
       </c>
       <c r="I103">
-        <v>7.7581343278406587E-2</v>
+        <v>7.4654907035614684E-2</v>
       </c>
       <c r="J103">
         <v>6977.7448180000001</v>
       </c>
       <c r="K103">
-        <v>6.3343693346281954E-2</v>
+        <v>6.1631735534879002E-2</v>
       </c>
       <c r="L103">
         <v>1.75</v>
@@ -13738,13 +13739,13 @@
         <v>3912.3106440000001</v>
       </c>
       <c r="I104">
-        <v>7.7983999999999998E-2</v>
+        <v>7.4566341568943414E-2</v>
       </c>
       <c r="J104">
         <v>7063.5350340200002</v>
       </c>
       <c r="K104">
-        <v>6.4260695561620507E-2</v>
+        <v>6.1818222205465082E-2</v>
       </c>
       <c r="L104">
         <v>2</v>
@@ -13833,13 +13834,13 @@
         <v>4272.7485489999999</v>
       </c>
       <c r="I105">
-        <v>7.6489000000000001E-2</v>
+        <v>7.3351270610501937E-2</v>
       </c>
       <c r="J105">
         <v>7200.5011758100009</v>
       </c>
       <c r="K105">
-        <v>6.359464072005909E-2</v>
+        <v>6.1571566386233158E-2</v>
       </c>
       <c r="L105">
         <v>2.5</v>
@@ -13928,13 +13929,13 @@
         <v>4662.773099</v>
       </c>
       <c r="I106">
-        <v>7.2753999999999999E-2</v>
+        <v>7.0779903855549803E-2</v>
       </c>
       <c r="J106">
         <v>7361.6614523999997</v>
       </c>
       <c r="K106">
-        <v>6.081645249579367E-2</v>
+        <v>5.9958698188727788E-2</v>
       </c>
       <c r="L106">
         <v>3</v>
@@ -14023,13 +14024,13 @@
         <v>5094.0788284</v>
       </c>
       <c r="I107">
-        <v>7.2019425558287081E-2</v>
+        <v>7.0165525725680633E-2</v>
       </c>
       <c r="J107">
         <v>7555.5404244999991</v>
       </c>
       <c r="K107">
-        <v>6.0680989218629001E-2</v>
+        <v>5.9936106830800417E-2</v>
       </c>
       <c r="L107">
         <v>3</v>
@@ -14118,13 +14119,13 @@
         <v>5236.3632733799996</v>
       </c>
       <c r="I108">
-        <v>6.7442347142971384E-2</v>
+        <v>6.8067711598639391E-2</v>
       </c>
       <c r="J108">
         <v>7759.8427391699997</v>
       </c>
       <c r="K108">
-        <v>5.7646178154100877E-2</v>
+        <v>5.8615900680145591E-2</v>
       </c>
       <c r="L108">
         <v>3</v>
@@ -14213,13 +14214,13 @@
         <v>5303.6694754800001</v>
       </c>
       <c r="I109">
-        <v>6.2280697122458831E-2</v>
+        <v>6.8307685699038043E-2</v>
       </c>
       <c r="J109">
         <v>7884.1293225199997</v>
       </c>
       <c r="K109">
-        <v>5.2975520346551307E-2</v>
+        <v>5.8280310354830972E-2</v>
       </c>
       <c r="L109">
         <v>3</v>
@@ -14403,13 +14404,13 @@
         <v>5368.7569914599999</v>
       </c>
       <c r="I111">
-        <v>6.7318458416892338E-2</v>
+        <v>6.5276745033706993E-2</v>
       </c>
       <c r="J111">
         <v>8007.8663106399999</v>
       </c>
       <c r="K111">
-        <v>5.6924602395562261E-2</v>
+        <v>5.5525343390765813E-2</v>
       </c>
       <c r="L111">
         <v>3.5</v>
@@ -14498,13 +14499,13 @@
         <v>5477.4377836900003</v>
       </c>
       <c r="I112">
-        <v>6.4512947592432035E-2</v>
+        <v>6.1866473987705617E-2</v>
       </c>
       <c r="J112">
         <v>8179.8068875700001</v>
       </c>
       <c r="K112">
-        <v>5.3989290813342659E-2</v>
+        <v>5.220357785208031E-2</v>
       </c>
       <c r="L112">
         <v>3.75</v>
@@ -14593,13 +14594,13 @@
         <v>5551.0687348299998</v>
       </c>
       <c r="I113">
-        <v>6.6532089446611847E-2</v>
+        <v>6.2430657423384717E-2</v>
       </c>
       <c r="J113">
         <v>8284.2491023999992</v>
       </c>
       <c r="K113">
-        <v>5.5145439826000772E-2</v>
+        <v>5.2433244629997662E-2</v>
       </c>
       <c r="L113">
         <v>4</v>
@@ -14688,13 +14689,13 @@
         <v>5633.5485502800002</v>
       </c>
       <c r="I114">
-        <v>6.7605010256114789E-2</v>
+        <v>6.3256836959660542E-2</v>
       </c>
       <c r="J114">
         <v>8398.7586886900008</v>
       </c>
       <c r="K114">
-        <v>5.5775217907000671E-2</v>
+        <v>5.2755879661456388E-2</v>
       </c>
       <c r="L114">
         <v>4.25</v>
@@ -14783,13 +14784,13 @@
         <v>5662.8610547999997</v>
       </c>
       <c r="I115">
-        <v>6.5429692347110907E-2</v>
+        <v>6.2503256104319005E-2</v>
       </c>
       <c r="J115">
         <v>8462.9789149700009</v>
       </c>
       <c r="K115">
-        <v>5.4037418553774218E-2</v>
+        <v>5.2325460742371259E-2</v>
       </c>
       <c r="L115">
         <v>4.25</v>
@@ -14878,13 +14879,13 @@
         <v>5725.6008683399996</v>
       </c>
       <c r="I116">
-        <v>6.8259452767847353E-2</v>
+        <v>6.484179433679077E-2</v>
       </c>
       <c r="J116">
         <v>8553.0507401600007</v>
       </c>
       <c r="K116">
-        <v>5.6358446599251967E-2</v>
+        <v>5.3915973243096542E-2</v>
       </c>
       <c r="L116">
         <v>4.25</v>
@@ -14973,13 +14974,13 @@
         <v>5812.0590015899998</v>
       </c>
       <c r="I117">
-        <v>6.8035515496629256E-2</v>
+        <v>6.4897786107131192E-2</v>
       </c>
       <c r="J117">
         <v>8679.5502381700007</v>
       </c>
       <c r="K117">
-        <v>5.5932153848833037E-2</v>
+        <v>5.3909079515007112E-2</v>
       </c>
       <c r="L117">
         <v>4.25</v>
@@ -15068,13 +15069,13 @@
         <v>5921.3550723699991</v>
       </c>
       <c r="I118">
-        <v>6.5547174451852833E-2</v>
+        <v>6.3573078307402636E-2</v>
       </c>
       <c r="J118">
         <v>8868.6136846999998</v>
       </c>
       <c r="K118">
-        <v>5.3490968163199148E-2</v>
+        <v>5.2633213856133267E-2</v>
       </c>
       <c r="L118">
         <v>4.25</v>
@@ -15163,13 +15164,13 @@
         <v>6041.26420745</v>
       </c>
       <c r="I119">
-        <v>6.6366218040186303E-2</v>
+        <v>6.4512318207579855E-2</v>
       </c>
       <c r="J119">
         <v>9033.4428496799992</v>
       </c>
       <c r="K119">
-        <v>5.4234600628192943E-2</v>
+        <v>5.3489718240364373E-2</v>
       </c>
       <c r="L119">
         <v>4.25</v>
@@ -15258,13 +15259,13 @@
         <v>6175.7699421699999</v>
       </c>
       <c r="I120">
-        <v>6.3509541715892404E-2</v>
+        <v>6.413490617156041E-2</v>
       </c>
       <c r="J120">
         <v>9235.2566162600015</v>
       </c>
       <c r="K120">
-        <v>5.2134360129451662E-2</v>
+        <v>5.3104082655496383E-2</v>
       </c>
       <c r="L120">
         <v>4.25</v>
@@ -15353,13 +15354,13 @@
         <v>6246.67535013</v>
       </c>
       <c r="I121">
-        <v>5.9607177234246869E-2</v>
+        <v>6.5634165810826081E-2</v>
       </c>
       <c r="J121">
         <v>9357.5380726099993</v>
       </c>
       <c r="K121">
-        <v>4.8885534219622877E-2</v>
+        <v>5.4190324227902542E-2</v>
       </c>
       <c r="L121">
         <v>4.25</v>
@@ -15543,13 +15544,13 @@
         <v>6242.1498302399996</v>
       </c>
       <c r="I123">
-        <v>6.6971716579883309E-2</v>
+        <v>6.4930003196697963E-2</v>
       </c>
       <c r="J123">
         <v>9397.9161654300005</v>
       </c>
       <c r="K123">
-        <v>5.4635975170619799E-2</v>
+        <v>5.3236716165823338E-2</v>
       </c>
       <c r="L123">
         <v>4.25</v>
@@ -15638,13 +15639,13 @@
         <v>6315.9264734600001</v>
       </c>
       <c r="I124">
-        <v>6.7102095415595725E-2</v>
+        <v>6.4455621810869307E-2</v>
       </c>
       <c r="J124">
         <v>9508.0005661399991</v>
       </c>
       <c r="K124">
-        <v>5.4673782877259637E-2</v>
+        <v>5.2888069915997288E-2</v>
       </c>
       <c r="L124">
         <v>4.25</v>
@@ -15733,13 +15734,13 @@
         <v>6380.6189163999998</v>
       </c>
       <c r="I125">
-        <v>7.081632760869204E-2</v>
+        <v>6.6714895585464909E-2</v>
       </c>
       <c r="J125">
         <v>9599.1133784600006</v>
       </c>
       <c r="K125">
-        <v>5.764421784950019E-2</v>
+        <v>5.4932022653497073E-2</v>
       </c>
       <c r="L125">
         <v>4.25</v>
@@ -15828,13 +15829,13 @@
         <v>6492.0052267400006</v>
       </c>
       <c r="I126">
-        <v>7.0871668484629613E-2</v>
+        <v>6.6523495188175366E-2</v>
       </c>
       <c r="J126">
         <v>9766.9052314199998</v>
       </c>
       <c r="K126">
-        <v>5.7617426489371522E-2</v>
+        <v>5.4598088243827239E-2</v>
       </c>
       <c r="L126">
         <v>4.25</v>
@@ -15923,13 +15924,13 @@
         <v>6524.0266904499986</v>
       </c>
       <c r="I127">
-        <v>7.0637726728584718E-2</v>
+        <v>6.7711290485792816E-2</v>
       </c>
       <c r="J127">
         <v>9816.3173731200004</v>
       </c>
       <c r="K127">
-        <v>5.7283712381772232E-2</v>
+        <v>5.5571754570369267E-2</v>
       </c>
       <c r="L127">
         <v>4.25</v>
@@ -16018,13 +16019,13 @@
         <v>6601.0925136100004</v>
       </c>
       <c r="I128">
-        <v>7.1638109347052073E-2</v>
+        <v>6.822045091599549E-2</v>
       </c>
       <c r="J128">
         <v>9922.1421894800005</v>
       </c>
       <c r="K128">
-        <v>5.8150057450470582E-2</v>
+        <v>5.5707584094315157E-2</v>
       </c>
       <c r="L128">
         <v>4.25</v>
@@ -16113,13 +16114,13 @@
         <v>6674.5198953299996</v>
       </c>
       <c r="I129">
-        <v>7.3835330203272154E-2</v>
+        <v>7.0697600813774089E-2</v>
       </c>
       <c r="J129">
         <v>10046.7969486</v>
       </c>
       <c r="K129">
-        <v>5.9292969046518859E-2</v>
+        <v>5.7269894712692927E-2</v>
       </c>
       <c r="L129">
         <v>4.25</v>
@@ -16208,13 +16209,13 @@
         <v>6763.7167086999998</v>
       </c>
       <c r="I130">
-        <v>7.2966914485816339E-2</v>
+        <v>7.0992818341366143E-2</v>
       </c>
       <c r="J130">
         <v>10186.77912967</v>
       </c>
       <c r="K130">
-        <v>5.8752494939918097E-2</v>
+        <v>5.7894740632852222E-2</v>
       </c>
       <c r="L130">
         <v>4.25</v>
@@ -16303,13 +16304,13 @@
         <v>6884.1508504399999</v>
       </c>
       <c r="I131">
-        <v>7.3578190288730472E-2</v>
+        <v>7.1724290456124024E-2</v>
       </c>
       <c r="J131">
         <v>10356.158876900001</v>
       </c>
       <c r="K131">
-        <v>5.9198036957261703E-2</v>
+        <v>5.8453154569433133E-2</v>
       </c>
       <c r="L131">
         <v>4.25</v>
@@ -16398,13 +16399,13 @@
         <v>7036.4793989500004</v>
       </c>
       <c r="I132">
-        <v>7.2414137036489412E-2</v>
+        <v>7.3039501492157419E-2</v>
       </c>
       <c r="J132">
         <v>10574.68853976</v>
       </c>
       <c r="K132">
-        <v>5.8488050435198648E-2</v>
+        <v>5.9457772961243362E-2</v>
       </c>
       <c r="L132">
         <v>4.25</v>
@@ -16493,13 +16494,13 @@
         <v>7017.5664852399996</v>
       </c>
       <c r="I133">
-        <v>6.2411303853150642E-2</v>
+        <v>6.8438292429729847E-2</v>
       </c>
       <c r="J133">
         <v>10578.21333837</v>
       </c>
       <c r="K133">
-        <v>5.0833170107236467E-2</v>
+        <v>5.6137960115516132E-2</v>
       </c>
       <c r="L133">
         <v>4.25</v>
@@ -16683,13 +16684,13 @@
         <v>7017.3563617300006</v>
       </c>
       <c r="I135">
-        <v>7.2982204606713286E-2</v>
+        <v>7.0940491223527941E-2</v>
       </c>
       <c r="J135">
         <v>10694.63997801</v>
       </c>
       <c r="K135">
-        <v>5.8438343810082352E-2</v>
+        <v>5.7039084805285897E-2</v>
       </c>
       <c r="L135">
         <v>4.25</v>
@@ -16778,13 +16779,13 @@
         <v>7056.9153317700002</v>
       </c>
       <c r="I136">
-        <v>7.4068874130717124E-2</v>
+        <v>7.1422400525990706E-2</v>
       </c>
       <c r="J136">
         <v>10732.69467635</v>
       </c>
       <c r="K136">
-        <v>5.9465296891036523E-2</v>
+        <v>5.7679583929774167E-2</v>
       </c>
       <c r="L136">
         <v>4.25</v>
@@ -16873,13 +16874,13 @@
         <v>7168.7382187100002</v>
       </c>
       <c r="I137">
-        <v>7.6681242934118307E-2</v>
+        <v>7.2579810910891177E-2</v>
       </c>
       <c r="J137">
         <v>10899.965093860001</v>
       </c>
       <c r="K137">
-        <v>6.0157095058897443E-2</v>
+        <v>5.7444899862894333E-2</v>
       </c>
       <c r="L137">
         <v>4.25</v>
@@ -16968,13 +16969,13 @@
         <v>7271.0032377099997</v>
       </c>
       <c r="I138">
-        <v>7.7914889924932174E-2</v>
+        <v>7.3566716628477927E-2</v>
       </c>
       <c r="J138">
         <v>11083.7092426</v>
       </c>
       <c r="K138">
-        <v>6.1098809124944441E-2</v>
+        <v>5.8079470879400158E-2</v>
       </c>
       <c r="L138">
         <v>4.25</v>
@@ -17063,13 +17064,13 @@
         <v>7316.0300982299996</v>
       </c>
       <c r="I139">
-        <v>7.47275816295873E-2</v>
+        <v>7.1801145386795398E-2</v>
       </c>
       <c r="J139">
         <v>11194.17080588</v>
       </c>
       <c r="K139">
-        <v>5.8431975136239662E-2</v>
+        <v>5.6720017324836697E-2</v>
       </c>
       <c r="L139">
         <v>4.25</v>
@@ -17158,13 +17159,13 @@
         <v>7345.4553875900001</v>
       </c>
       <c r="I140">
-        <v>7.8715717624105661E-2</v>
+        <v>7.5298059193049077E-2</v>
       </c>
       <c r="J140">
         <v>11242.5719955</v>
       </c>
       <c r="K140">
-        <v>6.193657816011449E-2</v>
+        <v>5.9494104803959072E-2</v>
       </c>
       <c r="L140">
         <v>4.25</v>
@@ -17253,13 +17254,13 @@
         <v>7399.3781635300002</v>
       </c>
       <c r="I141">
-        <v>8.234918440623494E-2</v>
+        <v>7.9211455016736876E-2</v>
       </c>
       <c r="J141">
         <v>11356.820464349999</v>
       </c>
       <c r="K141">
-        <v>6.4197216522761003E-2</v>
+        <v>6.2174142188935071E-2</v>
       </c>
       <c r="L141">
         <v>4.25</v>
@@ -17348,13 +17349,13 @@
         <v>7443.9502804599997</v>
       </c>
       <c r="I142">
-        <v>8.267117211884055E-2</v>
+        <v>8.0697075974390353E-2</v>
       </c>
       <c r="J142">
         <v>11449.76199483</v>
       </c>
       <c r="K142">
-        <v>6.3980959824386008E-2</v>
+        <v>6.3123205517320133E-2</v>
       </c>
       <c r="L142">
         <v>4.25</v>
@@ -17443,13 +17444,13 @@
         <v>7549.2751983099997</v>
       </c>
       <c r="I143">
-        <v>8.2441192761038257E-2</v>
+        <v>8.0587292928431808E-2</v>
       </c>
       <c r="J143">
         <v>11602.08688642</v>
       </c>
       <c r="K143">
-        <v>6.4066901897625719E-2</v>
+        <v>6.3322019509797142E-2</v>
       </c>
       <c r="L143">
         <v>4.25</v>
@@ -17538,13 +17539,13 @@
         <v>7646.1612642199998</v>
       </c>
       <c r="I144">
-        <v>7.507124213637098E-2</v>
+        <v>7.5696606592038987E-2</v>
       </c>
       <c r="J144">
         <v>11778.91175277</v>
       </c>
       <c r="K144">
-        <v>5.8152070917665097E-2</v>
+        <v>5.9121793443709811E-2</v>
       </c>
       <c r="L144">
         <v>4</v>
@@ -17633,13 +17634,13 @@
         <v>7704.6469238600002</v>
       </c>
       <c r="I145">
-        <v>7.1600772484668382E-2</v>
+        <v>7.7627761061247594E-2</v>
       </c>
       <c r="J145">
         <v>11900.02950861</v>
       </c>
       <c r="K145">
-        <v>5.5503418881618367E-2</v>
+        <v>6.0808208889898033E-2</v>
       </c>
       <c r="L145">
         <v>4</v>
@@ -17823,13 +17824,13 @@
         <v>7705.5992425499999</v>
       </c>
       <c r="I147">
-        <v>8.1318553987325931E-2</v>
+        <v>7.9276840604140586E-2</v>
       </c>
       <c r="J147">
         <v>11960.91661169</v>
       </c>
       <c r="K147">
-        <v>6.3389903627366823E-2</v>
+        <v>6.1990644622570368E-2</v>
       </c>
       <c r="L147">
         <v>4</v>
@@ -17918,13 +17919,13 @@
         <v>7760.0555636899999</v>
       </c>
       <c r="I148">
-        <v>8.2288951304409719E-2</v>
+        <v>7.9642477699683301E-2</v>
       </c>
       <c r="J148">
         <v>12064.83212861</v>
       </c>
       <c r="K148">
-        <v>6.431762274419657E-2</v>
+        <v>6.2531909782934214E-2</v>
       </c>
       <c r="L148">
         <v>4</v>
@@ -18013,13 +18014,13 @@
         <v>7808.2643688199996</v>
       </c>
       <c r="I149">
-        <v>8.5848862388262309E-2</v>
+        <v>8.1747430365035179E-2</v>
       </c>
       <c r="J149">
         <v>12155.796386980001</v>
       </c>
       <c r="K149">
-        <v>6.6814465065400758E-2</v>
+        <v>6.4102269869397641E-2</v>
       </c>
       <c r="L149">
         <v>4</v>
@@ -18108,13 +18109,13 @@
         <v>7812.9467608800014</v>
       </c>
       <c r="I150">
-        <v>8.8894841922840959E-2</v>
+        <v>8.4546668626386712E-2</v>
       </c>
       <c r="J150">
         <v>12192.01394854</v>
       </c>
       <c r="K150">
-        <v>6.9270128068639095E-2</v>
+        <v>6.6250789823094805E-2</v>
       </c>
       <c r="L150">
         <v>4</v>
@@ -18203,13 +18204,13 @@
         <v>7825.7836045800004</v>
       </c>
       <c r="I151">
-        <v>8.542578831195255E-2</v>
+        <v>8.2499352069160647E-2</v>
       </c>
       <c r="J151">
         <v>12244.055331310001</v>
       </c>
       <c r="K151">
-        <v>6.670947266314016E-2</v>
+        <v>6.4997514851737201E-2</v>
       </c>
       <c r="L151">
         <v>4</v>
@@ -18298,13 +18299,13 @@
         <v>7867.5535649099993</v>
       </c>
       <c r="I152">
-        <v>8.8087475002520413E-2</v>
+        <v>8.466981657146383E-2</v>
       </c>
       <c r="J152">
         <v>12298.53065982</v>
       </c>
       <c r="K152">
-        <v>6.8611855417560111E-2</v>
+        <v>6.6169382061404686E-2</v>
       </c>
       <c r="L152">
         <v>3.75</v>
@@ -18393,13 +18394,13 @@
         <v>7935.7251720700006</v>
       </c>
       <c r="I153">
-        <v>8.9387247466253719E-2</v>
+        <v>8.6249518076755655E-2</v>
       </c>
       <c r="J153">
         <v>12423.142105340001</v>
       </c>
       <c r="K153">
-        <v>6.9138200997540075E-2</v>
+        <v>6.7115126663714136E-2</v>
       </c>
       <c r="L153">
         <v>3.75</v>
@@ -18488,13 +18489,13 @@
         <v>7966.5615898699998</v>
       </c>
       <c r="I154">
-        <v>8.697806414891561E-2</v>
+        <v>8.5003968004465413E-2</v>
       </c>
       <c r="J154">
         <v>12500.12962673</v>
       </c>
       <c r="K154">
-        <v>6.7287672184726824E-2</v>
+        <v>6.6429917877660949E-2</v>
       </c>
       <c r="L154">
         <v>3.5</v>
@@ -18583,13 +18584,13 @@
         <v>8042.4083267100004</v>
       </c>
       <c r="I155">
-        <v>8.6612947532963239E-2</v>
+        <v>8.475904770035679E-2</v>
       </c>
       <c r="J155">
         <v>12636.29765122</v>
       </c>
       <c r="K155">
-        <v>6.6277931884513724E-2</v>
+        <v>6.5533049496685147E-2</v>
       </c>
       <c r="L155">
         <v>3.5</v>
@@ -18678,13 +18679,13 @@
         <v>8160.5943862800004</v>
       </c>
       <c r="I156">
-        <v>8.5645862839974177E-2</v>
+        <v>8.6271227295642183E-2</v>
       </c>
       <c r="J156">
         <v>12818.26374996</v>
       </c>
       <c r="K156">
-        <v>6.5795418081690815E-2</v>
+        <v>6.6765140607735529E-2</v>
       </c>
       <c r="L156">
         <v>3.5</v>
@@ -18773,13 +18774,13 @@
         <v>8153.8438916599998</v>
       </c>
       <c r="I157">
-        <v>7.353249876825102E-2</v>
+        <v>7.9559487344830232E-2</v>
       </c>
       <c r="J157">
         <v>12920.909428679999</v>
       </c>
       <c r="K157">
-        <v>5.6493854187210403E-2</v>
+        <v>6.1798644195490068E-2</v>
       </c>
       <c r="L157">
         <v>3.5</v>
@@ -18963,13 +18964,13 @@
         <v>8165.5200198800003</v>
       </c>
       <c r="I159">
-        <v>7.8446753359305774E-2</v>
+        <v>7.6405039976120429E-2</v>
       </c>
       <c r="J159">
         <v>13048.19116486</v>
       </c>
       <c r="K159">
-        <v>6.1651151752468297E-2</v>
+        <v>6.0251892747671842E-2</v>
       </c>
       <c r="L159">
         <v>3.25</v>
@@ -19058,13 +19059,13 @@
         <v>8258.6702812399999</v>
       </c>
       <c r="I160">
-        <v>7.9117605333421076E-2</v>
+        <v>7.6471131728694658E-2</v>
       </c>
       <c r="J160">
         <v>13169.101907710001</v>
       </c>
       <c r="K160">
-        <v>6.2258159132323937E-2</v>
+        <v>6.0472446171061588E-2</v>
       </c>
       <c r="L160">
         <v>3.25</v>
@@ -19153,13 +19154,13 @@
         <v>8340.3753127</v>
       </c>
       <c r="I161">
-        <v>8.064317190928226E-2</v>
+        <v>7.654173988605513E-2</v>
       </c>
       <c r="J161">
         <v>13316.859910970001</v>
       </c>
       <c r="K161">
-        <v>6.3701024068083784E-2</v>
+        <v>6.0988828872080673E-2</v>
       </c>
       <c r="L161">
         <v>3.25</v>
@@ -19248,13 +19249,13 @@
         <v>8410.5892563899997</v>
       </c>
       <c r="I162">
-        <v>8.3306582030227075E-2</v>
+        <v>7.8958408733772828E-2</v>
       </c>
       <c r="J162">
         <v>13411.963453320001</v>
       </c>
       <c r="K162">
-        <v>6.5697727036520034E-2</v>
+        <v>6.2678388790975745E-2</v>
       </c>
       <c r="L162">
         <v>3.25</v>
@@ -19343,13 +19344,13 @@
         <v>8379.84422051</v>
       </c>
       <c r="I163">
-        <v>8.0236210610497433E-2</v>
+        <v>7.730977436770553E-2</v>
       </c>
       <c r="J163">
         <v>13405.96638387</v>
       </c>
       <c r="K163">
-        <v>6.4001706796933913E-2</v>
+        <v>6.2289748985530947E-2</v>
       </c>
       <c r="L163">
         <v>3.25</v>
@@ -19438,13 +19439,13 @@
         <v>8341.8875228500001</v>
       </c>
       <c r="I164">
-        <v>7.6780871815348387E-2</v>
+        <v>7.3363213384291803E-2</v>
       </c>
       <c r="J164">
         <v>13422.44654836</v>
       </c>
       <c r="K164">
-        <v>6.2791279321054758E-2</v>
+        <v>6.0348805964899332E-2</v>
       </c>
       <c r="L164">
         <v>3.25</v>
@@ -19533,13 +19534,13 @@
         <v>8413.3321996600007</v>
       </c>
       <c r="I165">
-        <v>7.8434839593837485E-2</v>
+        <v>7.5297110204339421E-2</v>
       </c>
       <c r="J165">
         <v>13565.90701938</v>
       </c>
       <c r="K165">
-        <v>6.4099543021174391E-2</v>
+        <v>6.2076468687348459E-2</v>
       </c>
       <c r="L165">
         <v>3.25</v>
@@ -19628,13 +19629,13 @@
         <v>8488.3181081000002</v>
       </c>
       <c r="I166">
-        <v>7.8426325855383144E-2</v>
+        <v>7.6452229710932948E-2</v>
       </c>
       <c r="J166">
         <v>13717.747039559999</v>
       </c>
       <c r="K166">
-        <v>6.3616083377492513E-2</v>
+        <v>6.2758329070426638E-2</v>
       </c>
       <c r="L166">
         <v>3.5</v>
@@ -19723,13 +19724,13 @@
         <v>8598.0334791599998</v>
       </c>
       <c r="I167">
-        <v>7.8991143379026782E-2</v>
+        <v>7.7137243546420334E-2</v>
       </c>
       <c r="J167">
         <v>13874.0085726</v>
       </c>
       <c r="K167">
-        <v>6.3992446099059866E-2</v>
+        <v>6.3247563711231289E-2</v>
       </c>
       <c r="L167">
         <v>3.5</v>
@@ -19818,13 +19819,13 @@
         <v>8750.9560578100009</v>
       </c>
       <c r="I168">
-        <v>7.9373996844617795E-2</v>
+        <v>7.9999361300285801E-2</v>
       </c>
       <c r="J168">
         <v>14103.13868077</v>
       </c>
       <c r="K168">
-        <v>6.4166318992092047E-2</v>
+        <v>6.5136041518136761E-2</v>
       </c>
       <c r="L168">
         <v>3.5</v>
@@ -19913,13 +19914,13 @@
         <v>8795.2653784100003</v>
       </c>
       <c r="I169">
-        <v>7.0842996641067843E-2</v>
+        <v>7.6869985217647055E-2</v>
       </c>
       <c r="J169">
         <v>14253.83746105</v>
       </c>
       <c r="K169">
-        <v>5.7811171287153032E-2</v>
+        <v>6.3115961295432704E-2</v>
       </c>
       <c r="L169">
         <v>3.75</v>
@@ -20103,13 +20104,13 @@
         <v>8873.9178327999998</v>
       </c>
       <c r="I171">
-        <v>7.7052462962039062E-2</v>
+        <v>7.5010749578853717E-2</v>
       </c>
       <c r="J171">
         <v>14378.06269615</v>
       </c>
       <c r="K171">
-        <v>6.3286441188189616E-2</v>
+        <v>6.1887182183393161E-2</v>
       </c>
       <c r="L171">
         <v>4.25</v>
@@ -20198,13 +20199,13 @@
         <v>8949.0686506099992</v>
       </c>
       <c r="I172">
-        <v>7.7320678376160898E-2</v>
+        <v>7.467420477143448E-2</v>
       </c>
       <c r="J172">
         <v>14502.203805949999</v>
       </c>
       <c r="K172">
-        <v>6.3648538819409711E-2</v>
+        <v>6.1862825858147362E-2</v>
       </c>
       <c r="L172">
         <v>4.25</v>
@@ -20293,13 +20294,13 @@
         <v>9091.6101338799999</v>
       </c>
       <c r="I173">
-        <v>7.8239818606963246E-2</v>
+        <v>7.4138386583736116E-2</v>
       </c>
       <c r="J173">
         <v>14720.70087481</v>
       </c>
       <c r="K173">
-        <v>6.4129065655115045E-2</v>
+        <v>6.1416870459111927E-2</v>
       </c>
       <c r="L173">
         <v>4.25</v>
@@ -20388,13 +20389,13 @@
         <v>9192.7787757200003</v>
       </c>
       <c r="I174">
-        <v>7.837955164471655E-2</v>
+        <v>7.4031378348262303E-2</v>
       </c>
       <c r="J174">
         <v>14876.125973509999</v>
       </c>
       <c r="K174">
-        <v>6.6254236540822173E-2</v>
+        <v>6.3234898295277883E-2</v>
       </c>
       <c r="L174">
         <v>4.25</v>
@@ -20483,13 +20484,13 @@
         <v>9241.6136557400005</v>
       </c>
       <c r="I175">
-        <v>7.0491130159437129E-2</v>
+        <v>6.7564693916645227E-2</v>
       </c>
       <c r="J175">
         <v>14971.90514407</v>
       </c>
       <c r="K175">
-        <v>5.9552935284468381E-2</v>
+        <v>5.7840977473065422E-2</v>
       </c>
       <c r="L175">
         <v>4.25</v>
@@ -20578,13 +20579,13 @@
         <v>9365.434357099999</v>
       </c>
       <c r="I176">
-        <v>7.3095931681056409E-2</v>
+        <v>6.9678273249999825E-2</v>
       </c>
       <c r="J176">
         <v>15149.82843989</v>
       </c>
       <c r="K176">
-        <v>6.194730813511537E-2</v>
+        <v>5.9504834778959938E-2</v>
       </c>
       <c r="L176">
         <v>4.25</v>
@@ -20673,13 +20674,13 @@
         <v>9490.8248696200008</v>
       </c>
       <c r="I177">
-        <v>7.1772726712138094E-2</v>
+        <v>6.8634997322640029E-2</v>
       </c>
       <c r="J177">
         <v>15348.41417263</v>
       </c>
       <c r="K177">
-        <v>6.0962724324220403E-2</v>
+        <v>5.8939649990394472E-2</v>
       </c>
       <c r="L177">
         <v>4.25</v>
@@ -20768,13 +20769,13 @@
         <v>9692.5291187500006</v>
       </c>
       <c r="I178">
-        <v>7.0486646892643876E-2</v>
+        <v>6.8512550748193679E-2</v>
       </c>
       <c r="J178">
         <v>15637.098635099999</v>
       </c>
       <c r="K178">
-        <v>5.9605462619379282E-2</v>
+        <v>5.87477083123134E-2</v>
       </c>
       <c r="L178">
         <v>4.25</v>
@@ -20863,13 +20864,13 @@
         <v>9915.93192275</v>
       </c>
       <c r="I179">
-        <v>7.1044159059194978E-2</v>
+        <v>6.919025922658853E-2</v>
       </c>
       <c r="J179">
         <v>15972.12165134</v>
       </c>
       <c r="K179">
-        <v>5.943941305946359E-2</v>
+        <v>5.8694530671635013E-2</v>
       </c>
       <c r="L179">
         <v>4.25</v>
@@ -20958,13 +20959,13 @@
         <v>10190.416776829999</v>
       </c>
       <c r="I180">
-        <v>6.9813101719997328E-2</v>
+        <v>7.0438466175665335E-2</v>
       </c>
       <c r="J180">
         <v>16358.422680449999</v>
       </c>
       <c r="K180">
-        <v>5.8479990648076588E-2</v>
+        <v>5.9449713174121302E-2</v>
       </c>
       <c r="L180">
         <v>4.25</v>
@@ -21053,13 +21054,13 @@
         <v>10387.254654480001</v>
       </c>
       <c r="I181">
-        <v>6.2656671142581277E-2</v>
+        <v>6.8683659719160489E-2</v>
       </c>
       <c r="J181">
         <v>16795.659930760001</v>
       </c>
       <c r="K181">
-        <v>5.2602348724741177E-2</v>
+        <v>5.7907138733020842E-2</v>
       </c>
       <c r="L181">
         <v>4.25</v>
@@ -21243,13 +21244,13 @@
         <v>10569.4355805</v>
       </c>
       <c r="I183">
-        <v>6.8757529592287023E-2</v>
+        <v>6.6715816209101678E-2</v>
       </c>
       <c r="J183">
         <v>17083.45255469</v>
       </c>
       <c r="K183">
-        <v>5.834539881731108E-2</v>
+        <v>5.6946139812514618E-2</v>
       </c>
       <c r="L183">
         <v>4.25</v>
@@ -21338,13 +21339,13 @@
         <v>10646.158185439999</v>
       </c>
       <c r="I184">
-        <v>6.7487169501446384E-2</v>
+        <v>6.4840695896719966E-2</v>
       </c>
       <c r="J184">
         <v>17223.034069379999</v>
       </c>
       <c r="K184">
-        <v>5.6374563719651993E-2</v>
+        <v>5.4588850758389637E-2</v>
       </c>
       <c r="L184">
         <v>4.25</v>
@@ -21433,13 +21434,13 @@
         <v>10760.231230859999</v>
       </c>
       <c r="I185">
-        <v>6.9622029747972713E-2</v>
+        <v>6.5520597724745583E-2</v>
       </c>
       <c r="J185">
         <v>17445.65903757</v>
       </c>
       <c r="K185">
-        <v>5.7750206460548417E-2</v>
+        <v>5.50380112645453E-2</v>
       </c>
       <c r="L185">
         <v>4.25</v>
@@ -21528,13 +21529,13 @@
         <v>10908.338701979999</v>
       </c>
       <c r="I186">
-        <v>6.9124602944638444E-2</v>
+        <v>6.4776429648184197E-2</v>
       </c>
       <c r="J186">
         <v>17676.777908100001</v>
       </c>
       <c r="K186">
-        <v>5.7646148125958301E-2</v>
+        <v>5.4626809880414018E-2</v>
       </c>
       <c r="L186">
         <v>4</v>
@@ -21623,13 +21624,13 @@
         <v>11002.445870109999</v>
       </c>
       <c r="I187">
-        <v>6.8114731201354889E-2</v>
+        <v>6.5188294958562987E-2</v>
       </c>
       <c r="J187">
         <v>17846.44783605</v>
       </c>
       <c r="K187">
-        <v>5.650053750826288E-2</v>
+        <v>5.4788579696859921E-2</v>
       </c>
       <c r="L187">
         <v>4</v>
@@ -21718,13 +21719,13 @@
         <v>11127.4638713</v>
       </c>
       <c r="I188">
-        <v>6.8871025652718451E-2</v>
+        <v>6.5453367221661868E-2</v>
       </c>
       <c r="J188">
         <v>18080.77838353</v>
       </c>
       <c r="K188">
-        <v>5.737655985236742E-2</v>
+        <v>5.4934086496212002E-2</v>
       </c>
       <c r="L188">
         <v>3.75</v>
@@ -21813,13 +21814,13 @@
         <v>11257.6521689</v>
       </c>
       <c r="I189">
-        <v>6.9072175761314136E-2</v>
+        <v>6.5934446371816072E-2</v>
       </c>
       <c r="J189">
         <v>18294.073296750001</v>
       </c>
       <c r="K189">
-        <v>5.7090810808959933E-2</v>
+        <v>5.5067736475134001E-2</v>
       </c>
       <c r="L189">
         <v>3.75</v>
@@ -21908,13 +21909,13 @@
         <v>11416.66105242</v>
       </c>
       <c r="I190">
-        <v>6.8221201528524372E-2</v>
+        <v>6.6247105384074176E-2</v>
       </c>
       <c r="J190">
         <v>18591.994547769998</v>
       </c>
       <c r="K190">
-        <v>5.6205989351763193E-2</v>
+        <v>5.5348235044697311E-2</v>
       </c>
       <c r="L190">
         <v>3.5</v>
@@ -22003,13 +22004,13 @@
         <v>11578.39890303</v>
       </c>
       <c r="I191">
-        <v>7.0109487179403393E-2</v>
+        <v>6.8255587346796945E-2</v>
       </c>
       <c r="J191">
         <v>18792.029234900001</v>
       </c>
       <c r="K191">
-        <v>5.8052675730940313E-2</v>
+        <v>5.7307793343111743E-2</v>
       </c>
       <c r="L191">
         <v>3.5</v>
@@ -22098,13 +22099,13 @@
         <v>11766.68191992</v>
       </c>
       <c r="I192">
-        <v>6.8653966411075754E-2</v>
+        <v>6.927933086674376E-2</v>
       </c>
       <c r="J192">
         <v>19132.106648050001</v>
       </c>
       <c r="K192">
-        <v>5.6978414216142151E-2</v>
+        <v>5.7948136742186858E-2</v>
       </c>
       <c r="L192">
         <v>3.25</v>
@@ -22193,13 +22194,13 @@
         <v>11848.609286819999</v>
       </c>
       <c r="I193">
-        <v>6.4240339197165333E-2</v>
+        <v>7.0267327773744545E-2</v>
       </c>
       <c r="J193">
         <v>19318.403555860001</v>
       </c>
       <c r="K193">
-        <v>5.3468750441165371E-2</v>
+        <v>5.8773540449445043E-2</v>
       </c>
       <c r="L193">
         <v>3.25</v>
@@ -22383,13 +22384,13 @@
         <v>11926.22401939</v>
       </c>
       <c r="I195">
-        <v>7.2590843397915675E-2</v>
+        <v>7.054913001473033E-2</v>
       </c>
       <c r="J195">
         <v>19466.64535789</v>
       </c>
       <c r="K195">
-        <v>6.0116547653429171E-2</v>
+        <v>5.8717288648632723E-2</v>
       </c>
       <c r="L195">
         <v>3</v>
@@ -22478,13 +22479,13 @@
         <v>12008.959167860001</v>
       </c>
       <c r="I196">
-        <v>7.4555515021336255E-2</v>
+        <v>7.1909041416609837E-2</v>
       </c>
       <c r="J196">
         <v>19601.263714069999</v>
       </c>
       <c r="K196">
-        <v>6.2369318246173269E-2</v>
+        <v>6.058360528491092E-2</v>
       </c>
       <c r="L196">
         <v>2.75</v>
@@ -22573,13 +22574,13 @@
         <v>12121.904594170001</v>
       </c>
       <c r="I197">
-        <v>7.6127825750569367E-2</v>
+        <v>7.2026393727342236E-2</v>
       </c>
       <c r="J197">
         <v>19741.307738160001</v>
       </c>
       <c r="K197">
-        <v>6.3769613331975561E-2</v>
+        <v>6.1057418135972437E-2</v>
       </c>
       <c r="L197">
         <v>2.75</v>
@@ -22668,13 +22669,13 @@
         <v>12233.246765280001</v>
       </c>
       <c r="I198">
-        <v>7.5755453446768456E-2</v>
+        <v>7.1407280150314209E-2</v>
       </c>
       <c r="J198">
         <v>19860.186654410001</v>
       </c>
       <c r="K198">
-        <v>6.2921516471876465E-2</v>
+        <v>5.9902178226332183E-2</v>
       </c>
       <c r="L198">
         <v>2.75</v>
@@ -22763,13 +22764,13 @@
         <v>12263.66973541</v>
       </c>
       <c r="I199">
-        <v>7.6845529849756122E-2</v>
+        <v>7.391909360696422E-2</v>
       </c>
       <c r="J199">
         <v>19909.127866819999</v>
       </c>
       <c r="K199">
-        <v>6.4004678407519555E-2</v>
+        <v>6.2292720596116603E-2</v>
       </c>
       <c r="L199">
         <v>2.75</v>
@@ -22858,13 +22859,13 @@
         <v>12298.44860055</v>
       </c>
       <c r="I200">
-        <v>7.6506351751384441E-2</v>
+        <v>7.3088693320327858E-2</v>
       </c>
       <c r="J200">
         <v>19952.4820955</v>
       </c>
       <c r="K200">
-        <v>6.5021299340125502E-2</v>
+        <v>6.2578825983970077E-2</v>
       </c>
       <c r="L200">
         <v>2.75</v>
@@ -22953,13 +22954,13 @@
         <v>12379.50053367</v>
       </c>
       <c r="I201">
-        <v>7.9434811358134363E-2</v>
+        <v>7.6297081968636299E-2</v>
       </c>
       <c r="J201">
         <v>20086.543096689998</v>
       </c>
       <c r="K201">
-        <v>6.7474769600018511E-2</v>
+        <v>6.5451695266192572E-2</v>
       </c>
       <c r="L201">
         <v>2.75</v>
@@ -23048,13 +23049,13 @@
         <v>12466.49683412</v>
       </c>
       <c r="I202">
-        <v>7.9849397063619237E-2</v>
+        <v>7.7875300919169041E-2</v>
       </c>
       <c r="J202">
         <v>20267.926000790001</v>
       </c>
       <c r="K202">
-        <v>6.7620558061371433E-2</v>
+        <v>6.6762803754305558E-2</v>
       </c>
       <c r="L202">
         <v>2.75</v>
@@ -23143,13 +23144,13 @@
         <v>12610.14065913</v>
       </c>
       <c r="I203">
-        <v>8.1128799831371751E-2</v>
+        <v>7.9274899998765302E-2</v>
       </c>
       <c r="J203">
         <v>20501.550773080002</v>
       </c>
       <c r="K203">
-        <v>6.8974334205819637E-2</v>
+        <v>6.822945181799106E-2</v>
       </c>
       <c r="L203">
         <v>2.75</v>
@@ -23238,13 +23239,13 @@
         <v>12786.251230809999</v>
       </c>
       <c r="I204">
-        <v>7.7860896522282133E-2</v>
+        <v>7.848626097795014E-2</v>
       </c>
       <c r="J204">
         <v>20775.703495990001</v>
       </c>
       <c r="K204">
-        <v>6.6166789618716346E-2</v>
+        <v>6.713651214476106E-2</v>
       </c>
       <c r="L204">
         <v>2.75</v>
@@ -23333,13 +23334,13 @@
         <v>12916.139207509999</v>
       </c>
       <c r="I205">
-        <v>7.3988213223526472E-2</v>
+        <v>8.0015201800105684E-2</v>
       </c>
       <c r="J205">
         <v>20995.955960210002</v>
       </c>
       <c r="K205">
-        <v>6.3220582862030528E-2</v>
+        <v>6.8525372870310186E-2</v>
       </c>
       <c r="L205">
         <v>2.75</v>
@@ -23523,13 +23524,13 @@
         <v>13055.296494349999</v>
       </c>
       <c r="I207">
-        <v>7.9159943284877035E-2</v>
+        <v>7.711822990169169E-2</v>
       </c>
       <c r="J207">
         <v>21235.663027449998</v>
       </c>
       <c r="K207">
-        <v>7.0003918530275808E-2</v>
+        <v>6.8604659525479353E-2</v>
       </c>
       <c r="L207">
         <v>2.75</v>
@@ -23618,13 +23619,13 @@
         <v>13171.104831570001</v>
       </c>
       <c r="I208">
-        <v>7.8564969570335805E-2</v>
+        <v>7.5918495965609387E-2</v>
       </c>
       <c r="J208">
         <v>21431.423828319999</v>
       </c>
       <c r="K208">
-        <v>6.963390481401277E-2</v>
+        <v>6.7848191852750414E-2</v>
       </c>
       <c r="L208">
         <v>2.75</v>
@@ -23713,13 +23714,13 @@
         <v>13237.62139536</v>
       </c>
       <c r="I209">
-        <v>7.9644760796645203E-2</v>
+        <v>7.5543328773418073E-2</v>
       </c>
       <c r="J209">
         <v>21522.610524750002</v>
       </c>
       <c r="K209">
-        <v>7.1058283302636888E-2</v>
+        <v>6.8346088106633771E-2</v>
       </c>
       <c r="L209">
         <v>2.75</v>
@@ -23808,13 +23809,13 @@
         <v>13399.05141362</v>
       </c>
       <c r="I210">
-        <v>7.9215326131302652E-2</v>
+        <v>7.4867152834848405E-2</v>
       </c>
       <c r="J210">
         <v>21732.564350469998</v>
       </c>
       <c r="K210">
-        <v>7.0108722461325601E-2</v>
+        <v>6.7089384215781311E-2</v>
       </c>
       <c r="L210">
         <v>2.75</v>
@@ -23903,13 +23904,13 @@
         <v>13481.76974811</v>
       </c>
       <c r="I211">
-        <v>7.8112417201579382E-2</v>
+        <v>7.5185980958787479E-2</v>
       </c>
       <c r="J211">
         <v>21845.19135325</v>
       </c>
       <c r="K211">
-        <v>6.7683098282864423E-2</v>
+        <v>6.5971140471461465E-2</v>
       </c>
       <c r="L211">
         <v>2.75</v>
@@ -23998,13 +23999,13 @@
         <v>13605.61360875</v>
       </c>
       <c r="I212">
-        <v>8.0081950219377293E-2</v>
+        <v>7.666429178832071E-2</v>
       </c>
       <c r="J212">
         <v>21960.85232242</v>
       </c>
       <c r="K212">
-        <v>6.9730773316873315E-2</v>
+        <v>6.728829996071789E-2</v>
       </c>
       <c r="L212">
         <v>2.75</v>
@@ -24093,13 +24094,13 @@
         <v>13745.13069692</v>
       </c>
       <c r="I213">
-        <v>8.0054025885440749E-2</v>
+        <v>7.6916296495942685E-2</v>
       </c>
       <c r="J213">
         <v>22196.32818221</v>
       </c>
       <c r="K213">
-        <v>7.0166588965298482E-2</v>
+        <v>6.8143514631472557E-2</v>
       </c>
       <c r="L213">
         <v>2.5</v>
@@ -24188,13 +24189,13 @@
         <v>13850.034324</v>
       </c>
       <c r="I214">
-        <v>7.8926300858747259E-2</v>
+        <v>7.6952204714297062E-2</v>
       </c>
       <c r="J214">
         <v>22334.13241287</v>
       </c>
       <c r="K214">
-        <v>6.9038547814441797E-2</v>
+        <v>6.8180793507375922E-2</v>
       </c>
       <c r="L214">
         <v>2.5</v>
@@ -24283,13 +24284,13 @@
         <v>14071.466916949999</v>
       </c>
       <c r="I215">
-        <v>7.9211110938787188E-2</v>
+        <v>7.735721110618074E-2</v>
       </c>
       <c r="J215">
         <v>22629.592642719999</v>
       </c>
       <c r="K215">
-        <v>6.9359358750319192E-2</v>
+        <v>6.8614476362490615E-2</v>
       </c>
       <c r="L215">
         <v>2.5</v>
@@ -24378,13 +24379,13 @@
         <v>14350.546841380001</v>
       </c>
       <c r="I216">
-        <v>7.8888238414413905E-2</v>
+        <v>7.9513602870081912E-2</v>
       </c>
       <c r="J216">
         <v>22979.230807510001</v>
       </c>
       <c r="K216">
-        <v>6.9117154391039506E-2</v>
+        <v>7.008687691708422E-2</v>
       </c>
       <c r="L216">
         <v>2.25</v>
@@ -24473,13 +24474,13 @@
         <v>14482.16809841</v>
       </c>
       <c r="I217">
-        <v>7.4945273344062549E-2</v>
+        <v>8.0972261920641761E-2</v>
       </c>
       <c r="J217">
         <v>23211.904604250001</v>
       </c>
       <c r="K217">
-        <v>6.7060301519376114E-2</v>
+        <v>7.2365091527655773E-2</v>
       </c>
       <c r="L217">
         <v>2.25</v>
@@ -24663,13 +24664,13 @@
         <v>14643.50945086</v>
       </c>
       <c r="I219">
-        <v>7.9495365847674859E-2</v>
+        <v>7.7453652464489514E-2</v>
       </c>
       <c r="J219">
         <v>23449.600949539999</v>
       </c>
       <c r="K219">
-        <v>7.0814058522500112E-2</v>
+        <v>6.9414799517703657E-2</v>
       </c>
       <c r="L219">
         <v>2.25</v>
@@ -24758,13 +24759,13 @@
         <v>14310.29253604</v>
       </c>
       <c r="I220">
-        <v>7.9052390781736412E-2</v>
+        <v>7.6405917177009994E-2</v>
       </c>
       <c r="J220">
         <v>22869.881163869999</v>
       </c>
       <c r="K220">
-        <v>7.1529753897207393E-2</v>
+        <v>6.9744040935945037E-2</v>
       </c>
       <c r="L220">
         <v>1.25</v>
@@ -24853,13 +24854,13 @@
         <v>14089.046786409999</v>
       </c>
       <c r="I221">
-        <v>7.9516869480526817E-2</v>
+        <v>7.5415437457299686E-2</v>
       </c>
       <c r="J221">
         <v>22496.681269640001</v>
       </c>
       <c r="K221">
-        <v>7.1183401675834201E-2</v>
+        <v>6.8471206479831084E-2</v>
       </c>
       <c r="L221">
         <v>0.25</v>
@@ -24948,13 +24949,13 @@
         <v>14087.11798673</v>
       </c>
       <c r="I222">
-        <v>7.8700272163145985E-2</v>
+        <v>7.4352098866691738E-2</v>
       </c>
       <c r="J222">
         <v>22432.58766619</v>
       </c>
       <c r="K222">
-        <v>7.0627852643051409E-2</v>
+        <v>6.7608514397507119E-2</v>
       </c>
       <c r="L222">
         <v>0.25</v>
@@ -25043,13 +25044,13 @@
         <v>14248.5252177</v>
       </c>
       <c r="I223">
-        <v>7.7194744944105012E-2</v>
+        <v>7.426830870131311E-2</v>
       </c>
       <c r="J223">
         <v>22519.43442655</v>
       </c>
       <c r="K223">
-        <v>6.9934725827005356E-2</v>
+        <v>6.8222768015602397E-2</v>
       </c>
       <c r="L223">
         <v>0.25</v>
@@ -25138,13 +25139,13 @@
         <v>14932.27259633</v>
       </c>
       <c r="I224">
-        <v>6.9971061896284548E-2</v>
+        <v>6.6553403465227964E-2</v>
       </c>
       <c r="J224">
         <v>23167.214085669999</v>
       </c>
       <c r="K224">
-        <v>6.5361781476635739E-2</v>
+        <v>6.2919308120480313E-2</v>
       </c>
       <c r="L224">
         <v>0.25</v>
@@ -25233,13 +25234,13 @@
         <v>15448.824612799999</v>
       </c>
       <c r="I225">
-        <v>6.5903823177358822E-2</v>
+        <v>6.2766093787860758E-2</v>
       </c>
       <c r="J225">
         <v>23731.818671540001</v>
       </c>
       <c r="K225">
-        <v>6.2025704857388432E-2</v>
+        <v>6.00026305235625E-2</v>
       </c>
       <c r="L225">
         <v>0.25</v>
@@ -25328,13 +25329,13 @@
         <v>16164.727005320001</v>
       </c>
       <c r="I226">
-        <v>6.2153965633279233E-2</v>
+        <v>6.017986948882903E-2</v>
       </c>
       <c r="J226">
         <v>24518.274544330001</v>
       </c>
       <c r="K226">
-        <v>5.9501065340153432E-2</v>
+        <v>5.864331103308755E-2</v>
       </c>
       <c r="L226">
         <v>0.25</v>
@@ -25423,13 +25424,13 @@
         <v>16643.936121160001</v>
       </c>
       <c r="I227">
-        <v>5.7584737024525517E-2</v>
+        <v>5.5730837191919069E-2</v>
       </c>
       <c r="J227">
         <v>25086.317805409999</v>
       </c>
       <c r="K227">
-        <v>5.6220393512109917E-2</v>
+        <v>5.547551112428134E-2</v>
       </c>
       <c r="L227">
         <v>0.25</v>
@@ -25518,13 +25519,13 @@
         <v>17039.103716760001</v>
       </c>
       <c r="I228">
-        <v>5.4603099088178682E-2</v>
+        <v>5.5228463543846702E-2</v>
       </c>
       <c r="J228">
         <v>25677.110820710001</v>
       </c>
       <c r="K228">
-        <v>5.3677200989386442E-2</v>
+        <v>5.4646923515431163E-2</v>
       </c>
       <c r="L228">
         <v>0.25</v>
@@ -25613,13 +25614,13 @@
         <v>17303.47789563</v>
       </c>
       <c r="I229">
-        <v>4.9784130401181181E-2</v>
+        <v>5.5811118977760393E-2</v>
       </c>
       <c r="J229">
         <v>26089.69167837</v>
       </c>
       <c r="K229">
-        <v>4.9551879317600647E-2</v>
+        <v>5.4856669325880313E-2</v>
       </c>
       <c r="L229">
         <v>0.25</v>
@@ -25803,13 +25804,13 @@
         <v>17292.186950200001</v>
       </c>
       <c r="I231">
-        <v>5.8556908493768538E-2</v>
+        <v>5.6515195110583193E-2</v>
       </c>
       <c r="J231">
         <v>26134.26690708</v>
       </c>
       <c r="K231">
-        <v>5.5260045030716312E-2</v>
+        <v>5.3860786025919857E-2</v>
       </c>
       <c r="L231">
         <v>0.25</v>
@@ -25898,13 +25899,13 @@
         <v>17410.84239396</v>
       </c>
       <c r="I232">
-        <v>6.3918540870605292E-2</v>
+        <v>6.1272067265878867E-2</v>
       </c>
       <c r="J232">
         <v>26322.6821098</v>
       </c>
       <c r="K232">
-        <v>5.8415050610193427E-2</v>
+        <v>5.6629337648931077E-2</v>
       </c>
       <c r="L232">
         <v>0.25</v>
@@ -25993,13 +25994,13 @@
         <v>17590.599337340002</v>
       </c>
       <c r="I233">
-        <v>6.6101338952208197E-2</v>
+        <v>6.1999906928981073E-2</v>
       </c>
       <c r="J233">
         <v>26584.691770860001</v>
       </c>
       <c r="K233">
-        <v>6.0217424312766929E-2</v>
+        <v>5.7505229116763812E-2</v>
       </c>
       <c r="L233">
         <v>0.25</v>
@@ -26088,13 +26089,13 @@
         <v>17861.444640760001</v>
       </c>
       <c r="I234">
-        <v>6.6689788999582042E-2</v>
+        <v>6.2341615703127802E-2</v>
       </c>
       <c r="J234">
         <v>26885.48267967</v>
       </c>
       <c r="K234">
-        <v>6.1461035527158411E-2</v>
+        <v>5.8441697281614129E-2</v>
       </c>
       <c r="L234">
         <v>0.25</v>
@@ -26183,13 +26184,13 @@
         <v>18024.676300989999</v>
       </c>
       <c r="I235">
-        <v>6.267882312027695E-2</v>
+        <v>5.9752386877485048E-2</v>
       </c>
       <c r="J235">
         <v>27078.29926571</v>
       </c>
       <c r="K235">
-        <v>5.7972704250960252E-2</v>
+        <v>5.6260746439557287E-2</v>
       </c>
       <c r="L235">
         <v>0.25</v>
@@ -26278,13 +26279,13 @@
         <v>18214.69351021</v>
       </c>
       <c r="I236">
-        <v>6.5127595126157206E-2</v>
+        <v>6.1709936695100623E-2</v>
       </c>
       <c r="J236">
         <v>27255.03137493</v>
       </c>
       <c r="K236">
-        <v>6.0287407098030543E-2</v>
+        <v>5.7844933741875118E-2</v>
       </c>
       <c r="L236">
         <v>0.25</v>
@@ -26373,13 +26374,13 @@
         <v>18427.78186173</v>
       </c>
       <c r="I237">
-        <v>6.3027044009135183E-2</v>
+        <v>5.9889314619637118E-2</v>
       </c>
       <c r="J237">
         <v>27343.611330520002</v>
       </c>
       <c r="K237">
-        <v>5.8169047983602687E-2</v>
+        <v>5.6145973649776762E-2</v>
       </c>
       <c r="L237">
         <v>0.5</v>
@@ -26468,13 +26469,13 @@
         <v>18797.73941237</v>
       </c>
       <c r="I238">
-        <v>6.1177140654117099E-2</v>
+        <v>5.9203044509666902E-2</v>
       </c>
       <c r="J238">
         <v>27750.49222706</v>
       </c>
       <c r="K238">
-        <v>5.6933365038454462E-2</v>
+        <v>5.607561073138858E-2</v>
       </c>
       <c r="L238">
         <v>1</v>
@@ -26563,13 +26564,13 @@
         <v>19083.164364209999</v>
       </c>
       <c r="I239">
-        <v>6.1382550182132331E-2</v>
+        <v>5.9528650349525883E-2</v>
       </c>
       <c r="J239">
         <v>28134.098670740001</v>
       </c>
       <c r="K239">
-        <v>5.6706347481436388E-2</v>
+        <v>5.5961465093607811E-2</v>
       </c>
       <c r="L239">
         <v>1.5</v>
@@ -26658,13 +26659,13 @@
         <v>19422.658219389999</v>
       </c>
       <c r="I240">
-        <v>5.9420327775620327E-2</v>
+        <v>6.004569223128834E-2</v>
       </c>
       <c r="J240">
         <v>28565.92184305</v>
       </c>
       <c r="K240">
-        <v>5.499271148437309E-2</v>
+        <v>5.5962434010417797E-2</v>
       </c>
       <c r="L240">
         <v>2</v>
@@ -26753,13 +26754,13 @@
         <v>19628.150631429999</v>
       </c>
       <c r="I241">
-        <v>5.4190274307697628E-2</v>
+        <v>6.021726288427684E-2</v>
       </c>
       <c r="J241">
         <v>28935.97941213</v>
       </c>
       <c r="K241">
-        <v>4.9919099083422812E-2</v>
+        <v>5.5223889091702477E-2</v>
       </c>
       <c r="L241">
         <v>2.5</v>
@@ -26943,13 +26944,13 @@
         <v>19819.768310349999</v>
       </c>
       <c r="I243">
-        <v>6.09586301843437E-2</v>
+        <v>5.8916916801158348E-2</v>
       </c>
       <c r="J243">
         <v>29288.31076013</v>
       </c>
       <c r="K243">
-        <v>5.5457174495057507E-2</v>
+        <v>5.4057915490261052E-2</v>
       </c>
       <c r="L243">
         <v>3.5</v>
@@ -27038,13 +27039,13 @@
         <v>20139.74479144</v>
       </c>
       <c r="I244">
-        <v>6.1288311514484932E-2</v>
+        <v>5.8641837909758507E-2</v>
       </c>
       <c r="J244">
         <v>29722.529257099999</v>
       </c>
       <c r="K244">
-        <v>5.5757423287727863E-2</v>
+        <v>5.3971710326465507E-2</v>
       </c>
       <c r="L244">
         <v>4</v>
@@ -27133,13 +27134,13 @@
         <v>20322.691519280001</v>
       </c>
       <c r="I245">
-        <v>6.1166226027724493E-2</v>
+        <v>5.7064794004497363E-2</v>
       </c>
       <c r="J245">
         <v>30001.613608889998</v>
       </c>
       <c r="K245">
-        <v>5.5916290567881458E-2</v>
+        <v>5.320409537187834E-2</v>
       </c>
       <c r="L245">
         <v>4.5</v>
@@ -27228,13 +27229,13 @@
         <v>20483.47195363</v>
       </c>
       <c r="I246">
-        <v>5.9320679424401293E-2</v>
+        <v>5.4972506127947053E-2</v>
       </c>
       <c r="J246">
         <v>30317.818495570002</v>
       </c>
       <c r="K246">
-        <v>5.4912329069562227E-2</v>
+        <v>5.1892990824017937E-2</v>
       </c>
       <c r="L246">
         <v>5</v>
@@ -27323,13 +27324,13 @@
         <v>20658.609303699999</v>
       </c>
       <c r="I247">
-        <v>5.8381463019584218E-2</v>
+        <v>5.5455026776792322E-2</v>
       </c>
       <c r="J247">
         <v>30580.22079214</v>
       </c>
       <c r="K247">
-        <v>5.4227063829317558E-2</v>
+        <v>5.2515106017914599E-2</v>
       </c>
       <c r="L247">
         <v>5.5</v>
@@ -27418,13 +27419,13 @@
         <v>20863.02957418</v>
       </c>
       <c r="I248">
-        <v>5.9807626479340903E-2</v>
+        <v>5.638996804828432E-2</v>
       </c>
       <c r="J248">
         <v>30839.297492670001</v>
       </c>
       <c r="K248">
-        <v>5.5901234558269557E-2</v>
+        <v>5.3458761202114131E-2</v>
       </c>
       <c r="L248">
         <v>6</v>
@@ -27513,13 +27514,13 @@
         <v>21115.346774969999</v>
       </c>
       <c r="I249">
-        <v>6.0149252036226841E-2</v>
+        <v>5.7011522646728777E-2</v>
       </c>
       <c r="J249">
         <v>31190.616839679999</v>
       </c>
       <c r="K249">
-        <v>5.6105843720721811E-2</v>
+        <v>5.4082769386895879E-2</v>
       </c>
       <c r="L249">
         <v>6.5</v>
@@ -27608,13 +27609,13 @@
         <v>21407.916797350001</v>
       </c>
       <c r="I250">
-        <v>6.1088183416888257E-2</v>
+        <v>5.9114087272438047E-2</v>
       </c>
       <c r="J250">
         <v>31594.40712752</v>
       </c>
       <c r="K250">
-        <v>5.6435549268683501E-2</v>
+        <v>5.5577794961617619E-2</v>
       </c>
       <c r="L250">
         <v>6.75</v>
@@ -27703,13 +27704,13 @@
         <v>21706.975802270001</v>
       </c>
       <c r="I251">
-        <v>6.3164004349081995E-2</v>
+        <v>6.1310104516475547E-2</v>
       </c>
       <c r="J251">
         <v>31994.406581439998</v>
       </c>
       <c r="K251">
-        <v>5.8453273802080541E-2</v>
+        <v>5.7708391414251957E-2</v>
       </c>
       <c r="L251">
         <v>7</v>
@@ -27798,13 +27799,13 @@
         <v>22105.60582493</v>
       </c>
       <c r="I252">
-        <v>6.4014908517191979E-2</v>
+        <v>6.4640272972859986E-2</v>
       </c>
       <c r="J252">
         <v>32499.555740330001</v>
       </c>
       <c r="K252">
-        <v>5.8638773235139899E-2</v>
+        <v>5.9608495761184613E-2</v>
       </c>
       <c r="L252">
         <v>7.25</v>
@@ -27893,13 +27894,13 @@
         <v>22169.33574626</v>
       </c>
       <c r="I253">
-        <v>5.8095715359323653E-2</v>
+        <v>6.4122703935902858E-2</v>
       </c>
       <c r="J253">
         <v>32666.835766330001</v>
       </c>
       <c r="K253">
-        <v>5.3441397333297017E-2</v>
+        <v>5.8746187341576682E-2</v>
       </c>
       <c r="L253">
         <v>7.5</v>

</xml_diff>